<commit_message>
docs: 更新 daily check 历史 2026-08-26
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -454,27 +454,22 @@
         <v>tdk-schema-semantic</v>
       </c>
     </row>
-    <row r="2" xml:space="preserve">
+    <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-11 04:29:32</v>
+        <v>2026-08-26 03:31:22</v>
       </c>
       <c r="B2" t="str">
-        <v>成功</v>
+        <v>失败</v>
       </c>
       <c r="C2">
-        <v>292</v>
+        <v>0</v>
       </c>
       <c r="D2" t="str">
+        <v>spawnSync /bin/sh ETIMEDOUT</v>
+      </c>
+      <c r="E2" t="str">
         <v/>
       </c>
-      <c r="E2" t="str" xml:space="preserve">
-        <v xml:space="preserve">https://atomgit.com/openeuler/openEuler-portal/issues/185
-https://atomgit.com/openeuler/openEuler-portal/issues/249
-https://atomgit.com/openeuler/openEuler-portal/issues/252
-https://atomgit.com/openeuler/openEuler-portal/issues/254
-https://atomgit.com/openeuler/openEuler-portal/issues/251
-https://atomgit.com/openeuler/openEuler-portal/issues/255</v>
-      </c>
       <c r="F2">
         <v>0</v>
       </c>
@@ -485,7 +480,7 @@
         <v>0</v>
       </c>
       <c r="I2">
-        <v>260</v>
+        <v>0</v>
       </c>
       <c r="J2">
         <v>0</v>
@@ -506,7 +501,7 @@
         <v>0</v>
       </c>
       <c r="P2">
-        <v>32</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -569,7 +564,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-11 04:29:32</v>
+        <v>2026-08-26 03:31:22</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -677,7 +672,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-11 04:29:32</v>
+        <v>2026-08-26 03:31:22</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -783,21 +778,25 @@
         <v>tdk-schema-semantic</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-08-11 04:29:32</v>
+        <v>2026-08-26 03:31:22</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
-      <c r="E2" t="str">
-        <v/>
+      <c r="E2" t="str" xml:space="preserve">
+        <v xml:space="preserve">https://atomgit.com/opengauss/website/issues/333
+https://atomgit.com/opengauss/website/issues/355
+https://atomgit.com/opengauss/website/issues/356
+https://atomgit.com/opengauss/website/issues/357
+https://atomgit.com/opengauss/website/issues/334</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -827,10 +826,10 @@
         <v>0</v>
       </c>
       <c r="O2">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="P2">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -893,7 +892,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-11 04:29:32</v>
+        <v>2026-08-26 03:31:22</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1001,7 +1000,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-11 04:29:32</v>
+        <v>2026-08-26 03:31:22</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1109,13 +1108,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-08-11 04:29:32</v>
+        <v>2026-08-26 03:31:22</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1135,7 +1134,7 @@
         <v>18</v>
       </c>
       <c r="I2">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="J2">
         <v>0</v>
@@ -1219,13 +1218,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-08-11 04:29:32</v>
+        <v>2026-08-26 03:31:22</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>165</v>
+        <v>178</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1233,7 +1232,10 @@
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://atomgit.com/openUBMC/website/issues/151
 https://atomgit.com/openUBMC/website/issues/152
-https://atomgit.com/openUBMC/website/issues/153</v>
+https://atomgit.com/openUBMC/website/issues/153
+https://atomgit.com/openUBMC/website/issues/157
+https://atomgit.com/openUBMC/website/issues/154
+https://atomgit.com/openUBMC/website/issues/155</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1245,13 +1247,13 @@
         <v>2</v>
       </c>
       <c r="I2">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="L2">
         <v>0</v>
@@ -1266,7 +1268,7 @@
         <v>0</v>
       </c>
       <c r="P2">
-        <v>0</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -1329,13 +1331,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-08-11 04:29:32</v>
+        <v>2026-08-26 03:31:22</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1343,12 +1345,11 @@
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://atomgit.com/hifloat/hifloat-portal/issues/4
 https://atomgit.com/hifloat/hifloat-portal/issues/5
+https://atomgit.com/hifloat/hifloat-portal/issues/6
 https://atomgit.com/hifloat/hifloat-portal/issues/7
-https://atomgit.com/hifloat/hifloat-portal/issues/8
 https://atomgit.com/hifloat/hifloat-portal/issues/10
 https://atomgit.com/hifloat/hifloat-portal/issues/12
-https://atomgit.com/hifloat/hifloat-portal/issues/13
-https://atomgit.com/hifloat/hifloat-portal/issues/11</v>
+https://atomgit.com/hifloat/hifloat-portal/issues/13</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1363,7 +1364,7 @@
         <v>36</v>
       </c>
       <c r="J2">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K2">
         <v>1</v>
@@ -1375,7 +1376,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O2">
         <v>0</v>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-08-27
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,19 +456,19 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-26 03:31:22</v>
+        <v>2026-08-27 12:45:17</v>
       </c>
       <c r="B2" t="str">
-        <v>失败</v>
+        <v>成功</v>
       </c>
       <c r="C2">
-        <v>0</v>
+        <v>284</v>
       </c>
       <c r="D2" t="str">
-        <v>spawnSync /bin/sh ETIMEDOUT</v>
+        <v/>
       </c>
       <c r="E2" t="str">
-        <v/>
+        <v>https://atomgit.com/openeuler/openEuler-portal/issues/185</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -480,7 +480,7 @@
         <v>0</v>
       </c>
       <c r="I2">
-        <v>0</v>
+        <v>284</v>
       </c>
       <c r="J2">
         <v>0</v>
@@ -564,7 +564,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-26 03:31:22</v>
+        <v>2026-08-27 12:45:17</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -672,7 +672,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-26 03:31:22</v>
+        <v>2026-08-27 12:45:17</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -780,22 +780,19 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-08-26 03:31:22</v>
+        <v>2026-08-27 12:45:17</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
       <c r="E2" t="str" xml:space="preserve">
-        <v xml:space="preserve">https://atomgit.com/opengauss/website/issues/333
-https://atomgit.com/opengauss/website/issues/355
-https://atomgit.com/opengauss/website/issues/356
-https://atomgit.com/opengauss/website/issues/357
+        <v xml:space="preserve">https://atomgit.com/opengauss/website/issues/360
 https://atomgit.com/opengauss/website/issues/334</v>
       </c>
       <c r="F2">
@@ -823,10 +820,10 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="O2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P2">
         <v>10</v>
@@ -892,7 +889,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-26 03:31:22</v>
+        <v>2026-08-27 12:45:17</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1000,7 +997,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-26 03:31:22</v>
+        <v>2026-08-27 12:45:17</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1108,13 +1105,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-08-26 03:31:22</v>
+        <v>2026-08-27 12:45:17</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1122,7 +1119,9 @@
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://atomgit.com/mindspore/mindspore-portal/issues/186
 https://atomgit.com/mindspore/mindspore-portal/issues/187
-https://atomgit.com/mindspore/mindspore-portal/issues/188</v>
+https://atomgit.com/mindspore/mindspore-portal/issues/188
+https://atomgit.com/mindspore/mindspore-portal/issues/210
+https://atomgit.com/mindspore/mindspore-portal/issues/211</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1149,10 +1148,10 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O2">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="P2">
         <v>0</v>
@@ -1218,13 +1217,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-08-26 03:31:22</v>
+        <v>2026-08-27 12:45:17</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>178</v>
+        <v>171</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1232,10 +1231,7 @@
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://atomgit.com/openUBMC/website/issues/151
 https://atomgit.com/openUBMC/website/issues/152
-https://atomgit.com/openUBMC/website/issues/153
-https://atomgit.com/openUBMC/website/issues/157
-https://atomgit.com/openUBMC/website/issues/154
-https://atomgit.com/openUBMC/website/issues/155</v>
+https://atomgit.com/openUBMC/website/issues/153</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1331,13 +1327,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-08-26 03:31:22</v>
+        <v>2026-08-27 12:45:17</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1346,10 +1342,7 @@
         <v xml:space="preserve">https://atomgit.com/hifloat/hifloat-portal/issues/4
 https://atomgit.com/hifloat/hifloat-portal/issues/5
 https://atomgit.com/hifloat/hifloat-portal/issues/6
-https://atomgit.com/hifloat/hifloat-portal/issues/7
-https://atomgit.com/hifloat/hifloat-portal/issues/10
-https://atomgit.com/hifloat/hifloat-portal/issues/12
-https://atomgit.com/hifloat/hifloat-portal/issues/13</v>
+https://atomgit.com/hifloat/hifloat-portal/issues/7</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1364,7 +1357,7 @@
         <v>36</v>
       </c>
       <c r="J2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K2">
         <v>1</v>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-08-28
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,13 +456,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-27 12:45:17</v>
+        <v>2026-08-28 13:48:28</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>284</v>
+        <v>242</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -480,7 +480,7 @@
         <v>0</v>
       </c>
       <c r="I2">
-        <v>284</v>
+        <v>242</v>
       </c>
       <c r="J2">
         <v>0</v>
@@ -564,7 +564,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-27 12:45:17</v>
+        <v>2026-08-28 13:48:28</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -672,7 +672,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-27 12:45:17</v>
+        <v>2026-08-28 13:48:28</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -778,22 +778,21 @@
         <v>tdk-schema-semantic</v>
       </c>
     </row>
-    <row r="2" xml:space="preserve">
+    <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-27 12:45:17</v>
+        <v>2026-08-28 13:48:28</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
-      <c r="E2" t="str" xml:space="preserve">
-        <v xml:space="preserve">https://atomgit.com/opengauss/website/issues/360
-https://atomgit.com/opengauss/website/issues/334</v>
+      <c r="E2" t="str">
+        <v>https://atomgit.com/opengauss/website/issues/360</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -820,10 +819,10 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O2">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="P2">
         <v>10</v>
@@ -889,7 +888,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-27 12:45:17</v>
+        <v>2026-08-28 13:48:28</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -997,7 +996,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-27 12:45:17</v>
+        <v>2026-08-28 13:48:28</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1105,13 +1104,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-08-27 12:45:17</v>
+        <v>2026-08-28 13:48:28</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1119,9 +1118,7 @@
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://atomgit.com/mindspore/mindspore-portal/issues/186
 https://atomgit.com/mindspore/mindspore-portal/issues/187
-https://atomgit.com/mindspore/mindspore-portal/issues/188
-https://atomgit.com/mindspore/mindspore-portal/issues/210
-https://atomgit.com/mindspore/mindspore-portal/issues/211</v>
+https://atomgit.com/mindspore/mindspore-portal/issues/188</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1148,10 +1145,10 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O2">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="P2">
         <v>0</v>
@@ -1217,7 +1214,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-08-27 12:45:17</v>
+        <v>2026-08-28 13:48:28</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1327,7 +1324,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-08-27 12:45:17</v>
+        <v>2026-08-28 13:48:28</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1341,8 +1338,8 @@
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://atomgit.com/hifloat/hifloat-portal/issues/4
 https://atomgit.com/hifloat/hifloat-portal/issues/5
-https://atomgit.com/hifloat/hifloat-portal/issues/6
-https://atomgit.com/hifloat/hifloat-portal/issues/7</v>
+https://atomgit.com/hifloat/hifloat-portal/issues/7
+https://atomgit.com/hifloat/hifloat-portal/issues/8</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1357,7 +1354,7 @@
         <v>36</v>
       </c>
       <c r="J2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K2">
         <v>1</v>
@@ -1369,7 +1366,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O2">
         <v>0</v>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-08-29
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,7 +456,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-28 13:48:28</v>
+        <v>2026-08-29 08:48:30</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -564,7 +564,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-28 13:48:28</v>
+        <v>2026-08-29 08:48:30</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -672,7 +672,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-28 13:48:28</v>
+        <v>2026-08-29 08:48:30</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -780,7 +780,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-28 13:48:28</v>
+        <v>2026-08-29 08:48:30</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -888,7 +888,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-28 13:48:28</v>
+        <v>2026-08-29 08:48:30</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -996,7 +996,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-28 13:48:28</v>
+        <v>2026-08-29 08:48:30</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1104,7 +1104,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-08-28 13:48:28</v>
+        <v>2026-08-29 08:48:30</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1214,13 +1214,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-08-28 13:48:28</v>
+        <v>2026-08-29 08:48:30</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1240,13 +1240,13 @@
         <v>2</v>
       </c>
       <c r="I2">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="L2">
         <v>0</v>
@@ -1324,7 +1324,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-08-28 13:48:28</v>
+        <v>2026-08-29 08:48:30</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1338,8 +1338,8 @@
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://atomgit.com/hifloat/hifloat-portal/issues/4
 https://atomgit.com/hifloat/hifloat-portal/issues/5
-https://atomgit.com/hifloat/hifloat-portal/issues/7
-https://atomgit.com/hifloat/hifloat-portal/issues/8</v>
+https://atomgit.com/hifloat/hifloat-portal/issues/6
+https://atomgit.com/hifloat/hifloat-portal/issues/7</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1354,7 +1354,7 @@
         <v>36</v>
       </c>
       <c r="J2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K2">
         <v>1</v>
@@ -1366,7 +1366,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O2">
         <v>0</v>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-08-30
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,7 +456,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-29 08:48:30</v>
+        <v>2026-08-30 07:49:48</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -564,7 +564,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-29 08:48:30</v>
+        <v>2026-08-30 07:49:48</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -672,7 +672,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-29 08:48:30</v>
+        <v>2026-08-30 07:49:48</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -780,7 +780,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-29 08:48:30</v>
+        <v>2026-08-30 07:49:48</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -888,7 +888,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-29 08:48:30</v>
+        <v>2026-08-30 07:49:48</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -996,7 +996,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-29 08:48:30</v>
+        <v>2026-08-30 07:49:48</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1104,7 +1104,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-08-29 08:48:30</v>
+        <v>2026-08-30 07:49:48</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1214,13 +1214,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-08-29 08:48:30</v>
+        <v>2026-08-30 07:49:48</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1228,7 +1228,8 @@
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://atomgit.com/openUBMC/website/issues/151
 https://atomgit.com/openUBMC/website/issues/152
-https://atomgit.com/openUBMC/website/issues/153</v>
+https://atomgit.com/openUBMC/website/issues/153
+https://atomgit.com/openUBMC/website/issues/185</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1255,7 +1256,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -1324,13 +1325,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-08-29 08:48:30</v>
+        <v>2026-08-30 07:49:48</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1339,7 +1340,8 @@
         <v xml:space="preserve">https://atomgit.com/hifloat/hifloat-portal/issues/4
 https://atomgit.com/hifloat/hifloat-portal/issues/5
 https://atomgit.com/hifloat/hifloat-portal/issues/6
-https://atomgit.com/hifloat/hifloat-portal/issues/7</v>
+https://atomgit.com/hifloat/hifloat-portal/issues/7
+https://atomgit.com/hifloat/hifloat-portal/issues/8</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1354,7 +1356,7 @@
         <v>36</v>
       </c>
       <c r="J2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K2">
         <v>1</v>
@@ -1366,7 +1368,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O2">
         <v>0</v>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-08-31
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,7 +456,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-30 07:49:48</v>
+        <v>2026-08-31 08:04:07</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -564,7 +564,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-30 07:49:48</v>
+        <v>2026-08-31 08:04:07</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -672,7 +672,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-30 07:49:48</v>
+        <v>2026-08-31 08:04:07</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -780,13 +780,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-30 07:49:48</v>
+        <v>2026-08-31 08:04:07</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -819,7 +819,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -888,7 +888,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-30 07:49:48</v>
+        <v>2026-08-31 08:04:07</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -996,7 +996,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-30 07:49:48</v>
+        <v>2026-08-31 08:04:07</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1104,7 +1104,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-08-30 07:49:48</v>
+        <v>2026-08-31 08:04:07</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1214,13 +1214,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-08-30 07:49:48</v>
+        <v>2026-08-31 08:04:07</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1228,8 +1228,7 @@
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://atomgit.com/openUBMC/website/issues/151
 https://atomgit.com/openUBMC/website/issues/152
-https://atomgit.com/openUBMC/website/issues/153
-https://atomgit.com/openUBMC/website/issues/185</v>
+https://atomgit.com/openUBMC/website/issues/153</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1256,7 +1255,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -1325,13 +1324,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-08-30 07:49:48</v>
+        <v>2026-08-31 08:04:07</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1340,8 +1339,7 @@
         <v xml:space="preserve">https://atomgit.com/hifloat/hifloat-portal/issues/4
 https://atomgit.com/hifloat/hifloat-portal/issues/5
 https://atomgit.com/hifloat/hifloat-portal/issues/6
-https://atomgit.com/hifloat/hifloat-portal/issues/7
-https://atomgit.com/hifloat/hifloat-portal/issues/8</v>
+https://atomgit.com/hifloat/hifloat-portal/issues/7</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1356,7 +1354,7 @@
         <v>36</v>
       </c>
       <c r="J2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K2">
         <v>1</v>
@@ -1368,7 +1366,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O2">
         <v>0</v>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-09-01
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -454,21 +454,22 @@
         <v>tdk-schema-semantic</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-08-31 08:04:07</v>
+        <v>2026-09-01 07:27:33</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
-      <c r="E2" t="str">
-        <v>https://atomgit.com/openeuler/openEuler-portal/issues/185</v>
+      <c r="E2" t="str" xml:space="preserve">
+        <v xml:space="preserve">https://atomgit.com/openeuler/openEuler-portal/issues/283
+https://atomgit.com/openeuler/openEuler-portal/issues/284</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -495,7 +496,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -564,7 +565,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-31 08:04:07</v>
+        <v>2026-09-01 07:27:33</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -672,7 +673,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-31 08:04:07</v>
+        <v>2026-09-01 07:27:33</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -778,21 +779,22 @@
         <v>tdk-schema-semantic</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-08-31 08:04:07</v>
+        <v>2026-09-01 07:27:33</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>3</v>
+        <v>161</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
-      <c r="E2" t="str">
-        <v>https://atomgit.com/opengauss/website/issues/360</v>
+      <c r="E2" t="str" xml:space="preserve">
+        <v xml:space="preserve">https://atomgit.com/opengauss/website/issues/367
+https://atomgit.com/opengauss/website/issues/360</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -810,7 +812,7 @@
         <v>0</v>
       </c>
       <c r="K2">
-        <v>0</v>
+        <v>159</v>
       </c>
       <c r="L2">
         <v>0</v>
@@ -819,7 +821,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -888,7 +890,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-31 08:04:07</v>
+        <v>2026-09-01 07:27:33</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -996,7 +998,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-31 08:04:07</v>
+        <v>2026-09-01 07:27:33</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1104,7 +1106,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-08-31 08:04:07</v>
+        <v>2026-09-01 07:27:33</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1214,13 +1216,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-08-31 08:04:07</v>
+        <v>2026-09-01 07:27:33</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1240,13 +1242,13 @@
         <v>2</v>
       </c>
       <c r="I2">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="L2">
         <v>0</v>
@@ -1324,7 +1326,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-08-31 08:04:07</v>
+        <v>2026-09-01 07:27:33</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-09-02
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -454,22 +454,21 @@
         <v>tdk-schema-semantic</v>
       </c>
     </row>
-    <row r="2" xml:space="preserve">
+    <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-01 07:27:33</v>
+        <v>2026-09-02 07:00:57</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
-      <c r="E2" t="str" xml:space="preserve">
-        <v xml:space="preserve">https://atomgit.com/openeuler/openEuler-portal/issues/283
-https://atomgit.com/openeuler/openEuler-portal/issues/284</v>
+      <c r="E2" t="str">
+        <v>https://atomgit.com/openeuler/openEuler-portal/issues/283</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -496,7 +495,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -565,7 +564,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-01 07:27:33</v>
+        <v>2026-09-02 07:00:57</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -673,7 +672,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-01 07:27:33</v>
+        <v>2026-09-02 07:00:57</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -781,7 +780,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-01 07:27:33</v>
+        <v>2026-09-02 07:00:57</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -890,7 +889,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-01 07:27:33</v>
+        <v>2026-09-02 07:00:57</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -998,7 +997,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-01 07:27:33</v>
+        <v>2026-09-02 07:00:57</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1106,7 +1105,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-01 07:27:33</v>
+        <v>2026-09-02 07:00:57</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1216,7 +1215,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-01 07:27:33</v>
+        <v>2026-09-02 07:00:57</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1326,7 +1325,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-01 07:27:33</v>
+        <v>2026-09-02 07:00:57</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1340,8 +1339,8 @@
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://atomgit.com/hifloat/hifloat-portal/issues/4
 https://atomgit.com/hifloat/hifloat-portal/issues/5
-https://atomgit.com/hifloat/hifloat-portal/issues/6
-https://atomgit.com/hifloat/hifloat-portal/issues/7</v>
+https://atomgit.com/hifloat/hifloat-portal/issues/7
+https://atomgit.com/hifloat/hifloat-portal/issues/8</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1356,7 +1355,7 @@
         <v>36</v>
       </c>
       <c r="J2">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K2">
         <v>1</v>
@@ -1368,7 +1367,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O2">
         <v>0</v>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-09-03
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,7 +456,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-02 07:00:57</v>
+        <v>2026-09-03 06:52:12</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -564,7 +564,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-02 07:00:57</v>
+        <v>2026-09-03 06:52:12</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -672,7 +672,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-02 07:00:57</v>
+        <v>2026-09-03 06:52:12</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -780,13 +780,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-02 07:00:57</v>
+        <v>2026-09-03 06:52:12</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -820,7 +820,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -889,7 +889,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-02 07:00:57</v>
+        <v>2026-09-03 06:52:12</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -997,7 +997,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-02 07:00:57</v>
+        <v>2026-09-03 06:52:12</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1105,7 +1105,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-02 07:00:57</v>
+        <v>2026-09-03 06:52:12</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1215,7 +1215,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-02 07:00:57</v>
+        <v>2026-09-03 06:52:12</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1325,7 +1325,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-02 07:00:57</v>
+        <v>2026-09-03 06:52:12</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1339,8 +1339,8 @@
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://atomgit.com/hifloat/hifloat-portal/issues/4
 https://atomgit.com/hifloat/hifloat-portal/issues/5
-https://atomgit.com/hifloat/hifloat-portal/issues/7
-https://atomgit.com/hifloat/hifloat-portal/issues/8</v>
+https://atomgit.com/hifloat/hifloat-portal/issues/6
+https://atomgit.com/hifloat/hifloat-portal/issues/7</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1355,7 +1355,7 @@
         <v>36</v>
       </c>
       <c r="J2">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K2">
         <v>1</v>
@@ -1367,7 +1367,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O2">
         <v>0</v>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-09-04
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,7 +456,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-03 06:52:12</v>
+        <v>2026-09-04 07:12:13</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -564,7 +564,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-03 06:52:12</v>
+        <v>2026-09-04 07:12:13</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -672,7 +672,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-03 06:52:12</v>
+        <v>2026-09-04 07:12:13</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -780,13 +780,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-03 06:52:12</v>
+        <v>2026-09-04 07:12:13</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>160</v>
+        <v>165</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -820,7 +820,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -889,7 +889,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-03 06:52:12</v>
+        <v>2026-09-04 07:12:13</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -997,7 +997,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-03 06:52:12</v>
+        <v>2026-09-04 07:12:13</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1105,7 +1105,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-03 06:52:12</v>
+        <v>2026-09-04 07:12:13</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1215,13 +1215,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-03 06:52:12</v>
+        <v>2026-09-04 07:12:13</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1241,13 +1241,13 @@
         <v>2</v>
       </c>
       <c r="I2">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="L2">
         <v>0</v>
@@ -1325,7 +1325,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-03 06:52:12</v>
+        <v>2026-09-04 07:12:13</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-09-05
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,7 +456,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-04 07:12:13</v>
+        <v>2026-09-05 06:53:36</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -564,7 +564,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-04 07:12:13</v>
+        <v>2026-09-05 06:53:36</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -672,7 +672,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-04 07:12:13</v>
+        <v>2026-09-05 06:53:36</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -780,13 +780,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-04 07:12:13</v>
+        <v>2026-09-05 06:53:36</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>165</v>
+        <v>160</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -820,7 +820,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -889,7 +889,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-04 07:12:13</v>
+        <v>2026-09-05 06:53:36</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -997,7 +997,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-04 07:12:13</v>
+        <v>2026-09-05 06:53:36</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1105,7 +1105,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-04 07:12:13</v>
+        <v>2026-09-05 06:53:36</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1215,7 +1215,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-04 07:12:13</v>
+        <v>2026-09-05 06:53:36</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1325,13 +1325,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-04 07:12:13</v>
+        <v>2026-09-05 06:53:36</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1340,7 +1340,8 @@
         <v xml:space="preserve">https://atomgit.com/hifloat/hifloat-portal/issues/4
 https://atomgit.com/hifloat/hifloat-portal/issues/5
 https://atomgit.com/hifloat/hifloat-portal/issues/6
-https://atomgit.com/hifloat/hifloat-portal/issues/7</v>
+https://atomgit.com/hifloat/hifloat-portal/issues/7
+https://atomgit.com/hifloat/hifloat-portal/issues/8</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1355,7 +1356,7 @@
         <v>36</v>
       </c>
       <c r="J2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K2">
         <v>1</v>
@@ -1367,7 +1368,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O2">
         <v>0</v>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-09-06
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,7 +456,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-05 06:53:36</v>
+        <v>2026-09-06 06:49:28</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -564,7 +564,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-05 06:53:36</v>
+        <v>2026-09-06 06:49:28</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -672,7 +672,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-05 06:53:36</v>
+        <v>2026-09-06 06:49:28</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -780,13 +780,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-05 06:53:36</v>
+        <v>2026-09-06 06:49:28</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -820,7 +820,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -889,7 +889,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-05 06:53:36</v>
+        <v>2026-09-06 06:49:28</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -997,7 +997,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-05 06:53:36</v>
+        <v>2026-09-06 06:49:28</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1105,7 +1105,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-05 06:53:36</v>
+        <v>2026-09-06 06:49:28</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1215,13 +1215,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-05 06:53:36</v>
+        <v>2026-09-06 06:49:28</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1229,7 +1229,8 @@
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://atomgit.com/openUBMC/website/issues/151
 https://atomgit.com/openUBMC/website/issues/152
-https://atomgit.com/openUBMC/website/issues/153</v>
+https://atomgit.com/openUBMC/website/issues/153
+https://atomgit.com/openUBMC/website/issues/185</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1256,7 +1257,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -1325,13 +1326,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-05 06:53:36</v>
+        <v>2026-09-06 06:49:28</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1340,8 +1341,7 @@
         <v xml:space="preserve">https://atomgit.com/hifloat/hifloat-portal/issues/4
 https://atomgit.com/hifloat/hifloat-portal/issues/5
 https://atomgit.com/hifloat/hifloat-portal/issues/6
-https://atomgit.com/hifloat/hifloat-portal/issues/7
-https://atomgit.com/hifloat/hifloat-portal/issues/8</v>
+https://atomgit.com/hifloat/hifloat-portal/issues/7</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1368,7 +1368,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O2">
         <v>0</v>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-09-07
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,7 +456,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-06 06:49:28</v>
+        <v>2026-09-07 07:00:24</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -564,7 +564,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-06 06:49:28</v>
+        <v>2026-09-07 07:00:24</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -672,7 +672,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-06 06:49:28</v>
+        <v>2026-09-07 07:00:24</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -780,13 +780,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-06 06:49:28</v>
+        <v>2026-09-07 07:00:24</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -820,7 +820,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -889,7 +889,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-06 06:49:28</v>
+        <v>2026-09-07 07:00:24</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -997,7 +997,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-06 06:49:28</v>
+        <v>2026-09-07 07:00:24</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1105,7 +1105,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-06 06:49:28</v>
+        <v>2026-09-07 07:00:24</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1215,13 +1215,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-06 06:49:28</v>
+        <v>2026-09-07 07:00:24</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1229,8 +1229,7 @@
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://atomgit.com/openUBMC/website/issues/151
 https://atomgit.com/openUBMC/website/issues/152
-https://atomgit.com/openUBMC/website/issues/153
-https://atomgit.com/openUBMC/website/issues/185</v>
+https://atomgit.com/openUBMC/website/issues/153</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1257,7 +1256,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -1326,13 +1325,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-06 06:49:28</v>
+        <v>2026-09-07 07:00:24</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1341,7 +1340,8 @@
         <v xml:space="preserve">https://atomgit.com/hifloat/hifloat-portal/issues/4
 https://atomgit.com/hifloat/hifloat-portal/issues/5
 https://atomgit.com/hifloat/hifloat-portal/issues/6
-https://atomgit.com/hifloat/hifloat-portal/issues/7</v>
+https://atomgit.com/hifloat/hifloat-portal/issues/7
+https://atomgit.com/hifloat/hifloat-portal/issues/8</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1356,7 +1356,7 @@
         <v>36</v>
       </c>
       <c r="J2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K2">
         <v>1</v>
@@ -1368,7 +1368,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O2">
         <v>0</v>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-09-08
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,7 +456,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-07 07:00:24</v>
+        <v>2026-09-08 07:00:13</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -564,7 +564,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-07 07:00:24</v>
+        <v>2026-09-08 07:00:13</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -672,7 +672,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-07 07:00:24</v>
+        <v>2026-09-08 07:00:13</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -780,7 +780,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-07 07:00:24</v>
+        <v>2026-09-08 07:00:13</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -889,7 +889,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-07 07:00:24</v>
+        <v>2026-09-08 07:00:13</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -997,7 +997,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-07 07:00:24</v>
+        <v>2026-09-08 07:00:13</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1105,13 +1105,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-07 07:00:24</v>
+        <v>2026-09-08 07:00:13</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1131,7 +1131,7 @@
         <v>18</v>
       </c>
       <c r="I2">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="J2">
         <v>0</v>
@@ -1215,7 +1215,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-07 07:00:24</v>
+        <v>2026-09-08 07:00:13</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1325,13 +1325,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-07 07:00:24</v>
+        <v>2026-09-08 07:00:13</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1340,8 +1340,7 @@
         <v xml:space="preserve">https://atomgit.com/hifloat/hifloat-portal/issues/4
 https://atomgit.com/hifloat/hifloat-portal/issues/5
 https://atomgit.com/hifloat/hifloat-portal/issues/6
-https://atomgit.com/hifloat/hifloat-portal/issues/7
-https://atomgit.com/hifloat/hifloat-portal/issues/8</v>
+https://atomgit.com/hifloat/hifloat-portal/issues/7</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1356,7 +1355,7 @@
         <v>36</v>
       </c>
       <c r="J2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K2">
         <v>1</v>
@@ -1368,7 +1367,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O2">
         <v>0</v>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-09-09
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,7 +456,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-08 07:00:13</v>
+        <v>2026-09-09 07:14:38</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -564,7 +564,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-08 07:00:13</v>
+        <v>2026-09-09 07:14:38</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -672,7 +672,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-08 07:00:13</v>
+        <v>2026-09-09 07:14:38</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -780,13 +780,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-08 07:00:13</v>
+        <v>2026-09-09 07:14:38</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -820,7 +820,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -889,7 +889,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-08 07:00:13</v>
+        <v>2026-09-09 07:14:38</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -997,7 +997,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-08 07:00:13</v>
+        <v>2026-09-09 07:14:38</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1105,7 +1105,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-08 07:00:13</v>
+        <v>2026-09-09 07:14:38</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1215,7 +1215,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-08 07:00:13</v>
+        <v>2026-09-09 07:14:38</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1325,13 +1325,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-08 07:00:13</v>
+        <v>2026-09-09 07:14:38</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1340,7 +1340,8 @@
         <v xml:space="preserve">https://atomgit.com/hifloat/hifloat-portal/issues/4
 https://atomgit.com/hifloat/hifloat-portal/issues/5
 https://atomgit.com/hifloat/hifloat-portal/issues/6
-https://atomgit.com/hifloat/hifloat-portal/issues/7</v>
+https://atomgit.com/hifloat/hifloat-portal/issues/7
+https://atomgit.com/hifloat/hifloat-portal/issues/8</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1355,7 +1356,7 @@
         <v>36</v>
       </c>
       <c r="J2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K2">
         <v>1</v>
@@ -1367,7 +1368,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O2">
         <v>0</v>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-09-10
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,7 +456,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-09 07:14:38</v>
+        <v>2026-09-10 07:16:08</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -564,7 +564,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-09 07:14:38</v>
+        <v>2026-09-10 07:16:08</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -672,7 +672,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-09 07:14:38</v>
+        <v>2026-09-10 07:16:08</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -780,7 +780,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-09 07:14:38</v>
+        <v>2026-09-10 07:16:08</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -889,7 +889,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-09 07:14:38</v>
+        <v>2026-09-10 07:16:08</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -997,7 +997,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-09 07:14:38</v>
+        <v>2026-09-10 07:16:08</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1105,7 +1105,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-09 07:14:38</v>
+        <v>2026-09-10 07:16:08</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1215,7 +1215,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-09 07:14:38</v>
+        <v>2026-09-10 07:16:08</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1325,13 +1325,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-09 07:14:38</v>
+        <v>2026-09-10 07:16:08</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1356,7 +1356,7 @@
         <v>36</v>
       </c>
       <c r="J2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K2">
         <v>1</v>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-09-11
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,7 +456,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-10 07:16:08</v>
+        <v>2026-09-11 07:17:50</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -564,7 +564,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-10 07:16:08</v>
+        <v>2026-09-11 07:17:50</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -672,7 +672,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-10 07:16:08</v>
+        <v>2026-09-11 07:17:50</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -780,7 +780,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-10 07:16:08</v>
+        <v>2026-09-11 07:17:50</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -889,7 +889,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-10 07:16:08</v>
+        <v>2026-09-11 07:17:50</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -997,7 +997,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-10 07:16:08</v>
+        <v>2026-09-11 07:17:50</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1105,13 +1105,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-10 07:16:08</v>
+        <v>2026-09-11 07:17:50</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1128,10 +1128,10 @@
         <v>0</v>
       </c>
       <c r="H2">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="I2">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="J2">
         <v>0</v>
@@ -1215,13 +1215,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-10 07:16:08</v>
+        <v>2026-09-11 07:17:50</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1247,7 +1247,7 @@
         <v>0</v>
       </c>
       <c r="K2">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="L2">
         <v>0</v>
@@ -1325,13 +1325,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-10 07:16:08</v>
+        <v>2026-09-11 07:17:50</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1340,8 +1340,7 @@
         <v xml:space="preserve">https://atomgit.com/hifloat/hifloat-portal/issues/4
 https://atomgit.com/hifloat/hifloat-portal/issues/5
 https://atomgit.com/hifloat/hifloat-portal/issues/6
-https://atomgit.com/hifloat/hifloat-portal/issues/7
-https://atomgit.com/hifloat/hifloat-portal/issues/8</v>
+https://atomgit.com/hifloat/hifloat-portal/issues/7</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1368,7 +1367,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O2">
         <v>0</v>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-09-12
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,7 +456,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-11 07:17:50</v>
+        <v>2026-09-12 06:54:01</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -564,7 +564,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-11 07:17:50</v>
+        <v>2026-09-12 06:54:01</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -672,7 +672,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-11 07:17:50</v>
+        <v>2026-09-12 06:54:01</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -780,13 +780,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-11 07:17:50</v>
+        <v>2026-09-12 06:54:01</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -820,7 +820,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -889,7 +889,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-11 07:17:50</v>
+        <v>2026-09-12 06:54:01</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -997,7 +997,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-11 07:17:50</v>
+        <v>2026-09-12 06:54:01</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1105,13 +1105,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-11 07:17:50</v>
+        <v>2026-09-12 06:54:01</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1131,7 +1131,7 @@
         <v>20</v>
       </c>
       <c r="I2">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="J2">
         <v>0</v>
@@ -1215,13 +1215,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-11 07:17:50</v>
+        <v>2026-09-12 06:54:01</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1241,13 +1241,13 @@
         <v>2</v>
       </c>
       <c r="I2">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="L2">
         <v>0</v>
@@ -1325,13 +1325,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-11 07:17:50</v>
+        <v>2026-09-12 06:54:01</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1340,7 +1340,8 @@
         <v xml:space="preserve">https://atomgit.com/hifloat/hifloat-portal/issues/4
 https://atomgit.com/hifloat/hifloat-portal/issues/5
 https://atomgit.com/hifloat/hifloat-portal/issues/6
-https://atomgit.com/hifloat/hifloat-portal/issues/7</v>
+https://atomgit.com/hifloat/hifloat-portal/issues/7
+https://atomgit.com/hifloat/hifloat-portal/issues/8</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1355,7 +1356,7 @@
         <v>36</v>
       </c>
       <c r="J2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K2">
         <v>1</v>
@@ -1367,7 +1368,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O2">
         <v>0</v>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-09-13
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,7 +456,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-12 06:54:01</v>
+        <v>2026-09-13 07:08:51</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -564,7 +564,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-12 06:54:01</v>
+        <v>2026-09-13 07:08:51</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -672,7 +672,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-12 06:54:01</v>
+        <v>2026-09-13 07:08:51</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -780,13 +780,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-12 06:54:01</v>
+        <v>2026-09-13 07:08:51</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -820,7 +820,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -889,7 +889,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-12 06:54:01</v>
+        <v>2026-09-13 07:08:51</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -997,7 +997,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-12 06:54:01</v>
+        <v>2026-09-13 07:08:51</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1105,7 +1105,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-12 06:54:01</v>
+        <v>2026-09-13 07:08:51</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1215,7 +1215,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-12 06:54:01</v>
+        <v>2026-09-13 07:08:51</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1325,13 +1325,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-12 06:54:01</v>
+        <v>2026-09-13 07:08:51</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1356,7 +1356,7 @@
         <v>36</v>
       </c>
       <c r="J2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K2">
         <v>1</v>
@@ -1368,7 +1368,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O2">
         <v>0</v>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-09-14
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,7 +456,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-13 07:08:51</v>
+        <v>2026-09-14 07:41:53</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -564,7 +564,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-13 07:08:51</v>
+        <v>2026-09-14 07:41:53</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -672,7 +672,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-13 07:08:51</v>
+        <v>2026-09-14 07:41:53</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -780,7 +780,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-13 07:08:51</v>
+        <v>2026-09-14 07:41:53</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -889,7 +889,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-13 07:08:51</v>
+        <v>2026-09-14 07:41:53</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -997,7 +997,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-13 07:08:51</v>
+        <v>2026-09-14 07:41:53</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1105,7 +1105,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-13 07:08:51</v>
+        <v>2026-09-14 07:41:53</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1215,13 +1215,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-13 07:08:51</v>
+        <v>2026-09-14 07:41:53</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1229,7 +1229,8 @@
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://atomgit.com/openUBMC/website/issues/151
 https://atomgit.com/openUBMC/website/issues/152
-https://atomgit.com/openUBMC/website/issues/153</v>
+https://atomgit.com/openUBMC/website/issues/153
+https://atomgit.com/openUBMC/website/issues/185</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1256,7 +1257,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -1325,7 +1326,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-13 07:08:51</v>
+        <v>2026-09-14 07:41:53</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-09-15
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,7 +456,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-14 07:41:53</v>
+        <v>2026-09-15 07:21:38</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -564,7 +564,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-14 07:41:53</v>
+        <v>2026-09-15 07:21:38</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -672,7 +672,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-14 07:41:53</v>
+        <v>2026-09-15 07:21:38</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -780,13 +780,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-14 07:41:53</v>
+        <v>2026-09-15 07:21:38</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -820,7 +820,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -889,7 +889,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-14 07:41:53</v>
+        <v>2026-09-15 07:21:38</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -997,7 +997,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-14 07:41:53</v>
+        <v>2026-09-15 07:21:38</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1105,7 +1105,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-14 07:41:53</v>
+        <v>2026-09-15 07:21:38</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1215,13 +1215,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-14 07:41:53</v>
+        <v>2026-09-15 07:21:38</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1229,8 +1229,7 @@
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://atomgit.com/openUBMC/website/issues/151
 https://atomgit.com/openUBMC/website/issues/152
-https://atomgit.com/openUBMC/website/issues/153
-https://atomgit.com/openUBMC/website/issues/185</v>
+https://atomgit.com/openUBMC/website/issues/153</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1257,7 +1256,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -1326,7 +1325,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-14 07:41:53</v>
+        <v>2026-09-15 07:21:38</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1341,8 +1340,7 @@
         <v xml:space="preserve">https://atomgit.com/hifloat/hifloat-portal/issues/4
 https://atomgit.com/hifloat/hifloat-portal/issues/5
 https://atomgit.com/hifloat/hifloat-portal/issues/6
-https://atomgit.com/hifloat/hifloat-portal/issues/7
-https://atomgit.com/hifloat/hifloat-portal/issues/8</v>
+https://atomgit.com/hifloat/hifloat-portal/issues/7</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1357,7 +1355,7 @@
         <v>36</v>
       </c>
       <c r="J2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K2">
         <v>1</v>
@@ -1369,7 +1367,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O2">
         <v>0</v>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-09-16
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,7 +456,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-15 07:21:38</v>
+        <v>2026-09-16 07:11:30</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -564,7 +564,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-15 07:21:38</v>
+        <v>2026-09-16 07:11:30</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -672,7 +672,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-15 07:21:38</v>
+        <v>2026-09-16 07:11:30</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -780,13 +780,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-15 07:21:38</v>
+        <v>2026-09-16 07:11:30</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -820,7 +820,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -889,7 +889,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-15 07:21:38</v>
+        <v>2026-09-16 07:11:30</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -997,7 +997,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-15 07:21:38</v>
+        <v>2026-09-16 07:11:30</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1105,7 +1105,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-15 07:21:38</v>
+        <v>2026-09-16 07:11:30</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1215,13 +1215,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-15 07:21:38</v>
+        <v>2026-09-16 07:11:30</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1241,13 +1241,13 @@
         <v>2</v>
       </c>
       <c r="I2">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="L2">
         <v>0</v>
@@ -1325,7 +1325,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-15 07:21:38</v>
+        <v>2026-09-16 07:11:30</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1340,7 +1340,8 @@
         <v xml:space="preserve">https://atomgit.com/hifloat/hifloat-portal/issues/4
 https://atomgit.com/hifloat/hifloat-portal/issues/5
 https://atomgit.com/hifloat/hifloat-portal/issues/6
-https://atomgit.com/hifloat/hifloat-portal/issues/7</v>
+https://atomgit.com/hifloat/hifloat-portal/issues/7
+https://atomgit.com/hifloat/hifloat-portal/issues/8</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1355,7 +1356,7 @@
         <v>36</v>
       </c>
       <c r="J2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K2">
         <v>1</v>
@@ -1367,7 +1368,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O2">
         <v>0</v>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-09-17
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,7 +456,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-16 07:11:30</v>
+        <v>2026-09-17 07:16:15</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -564,7 +564,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-16 07:11:30</v>
+        <v>2026-09-17 07:16:15</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -672,7 +672,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-16 07:11:30</v>
+        <v>2026-09-17 07:16:15</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -780,13 +780,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-16 07:11:30</v>
+        <v>2026-09-17 07:16:15</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>160</v>
+        <v>165</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -820,7 +820,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -889,7 +889,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-16 07:11:30</v>
+        <v>2026-09-17 07:16:15</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -997,7 +997,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-16 07:11:30</v>
+        <v>2026-09-17 07:16:15</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1105,7 +1105,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-16 07:11:30</v>
+        <v>2026-09-17 07:16:15</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1215,7 +1215,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-16 07:11:30</v>
+        <v>2026-09-17 07:16:15</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1325,7 +1325,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-16 07:11:30</v>
+        <v>2026-09-17 07:16:15</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-09-18
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,7 +456,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-17 07:16:15</v>
+        <v>2026-09-18 07:19:57</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -564,7 +564,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-17 07:16:15</v>
+        <v>2026-09-18 07:19:57</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -672,7 +672,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-17 07:16:15</v>
+        <v>2026-09-18 07:19:57</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -780,13 +780,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-17 07:16:15</v>
+        <v>2026-09-18 07:19:57</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -820,7 +820,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -889,7 +889,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-17 07:16:15</v>
+        <v>2026-09-18 07:19:57</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -997,7 +997,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-17 07:16:15</v>
+        <v>2026-09-18 07:19:57</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1105,7 +1105,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-17 07:16:15</v>
+        <v>2026-09-18 07:19:57</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1215,13 +1215,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-17 07:16:15</v>
+        <v>2026-09-18 07:19:57</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>182</v>
+        <v>188</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1247,7 +1247,7 @@
         <v>0</v>
       </c>
       <c r="K2">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="L2">
         <v>0</v>
@@ -1325,13 +1325,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-17 07:16:15</v>
+        <v>2026-09-18 07:19:57</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>67</v>
+        <v>74</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1350,13 +1350,13 @@
         <v>0</v>
       </c>
       <c r="H2">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="I2">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="J2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K2">
         <v>1</v>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-09-19
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,7 +456,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-18 07:19:57</v>
+        <v>2026-09-19 07:18:32</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -564,7 +564,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-18 07:19:57</v>
+        <v>2026-09-19 07:18:32</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -672,7 +672,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-18 07:19:57</v>
+        <v>2026-09-19 07:18:32</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -780,13 +780,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-18 07:19:57</v>
+        <v>2026-09-19 07:18:32</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -820,7 +820,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -889,7 +889,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-18 07:19:57</v>
+        <v>2026-09-19 07:18:32</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -997,7 +997,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-18 07:19:57</v>
+        <v>2026-09-19 07:18:32</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1105,7 +1105,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-18 07:19:57</v>
+        <v>2026-09-19 07:18:32</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1215,7 +1215,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-18 07:19:57</v>
+        <v>2026-09-19 07:18:32</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1325,13 +1325,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-18 07:19:57</v>
+        <v>2026-09-19 07:18:32</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1356,7 +1356,7 @@
         <v>39</v>
       </c>
       <c r="J2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K2">
         <v>1</v>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-09-20
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,7 +456,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-19 07:18:32</v>
+        <v>2026-09-20 07:39:21</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -564,7 +564,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-19 07:18:32</v>
+        <v>2026-09-20 07:39:21</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -672,7 +672,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-19 07:18:32</v>
+        <v>2026-09-20 07:39:21</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -780,13 +780,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-19 07:18:32</v>
+        <v>2026-09-20 07:39:21</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -820,7 +820,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -889,7 +889,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-19 07:18:32</v>
+        <v>2026-09-20 07:39:21</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -997,7 +997,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-19 07:18:32</v>
+        <v>2026-09-20 07:39:21</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1105,13 +1105,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-19 07:18:32</v>
+        <v>2026-09-20 07:39:21</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1119,7 +1119,8 @@
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://atomgit.com/mindspore/mindspore-portal/issues/186
 https://atomgit.com/mindspore/mindspore-portal/issues/187
-https://atomgit.com/mindspore/mindspore-portal/issues/188</v>
+https://atomgit.com/mindspore/mindspore-portal/issues/188
+https://atomgit.com/mindspore/mindspore-portal/issues/234</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1146,7 +1147,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -1215,7 +1216,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-19 07:18:32</v>
+        <v>2026-09-20 07:39:21</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1325,7 +1326,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-19 07:18:32</v>
+        <v>2026-09-20 07:39:21</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-09-21
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -454,21 +454,22 @@
         <v>tdk-schema-semantic</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-20 07:39:21</v>
+        <v>2026-09-21 07:48:08</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
-      <c r="E2" t="str">
-        <v>https://atomgit.com/openeuler/openEuler-portal/issues/283</v>
+      <c r="E2" t="str" xml:space="preserve">
+        <v xml:space="preserve">https://atomgit.com/openeuler/openEuler-portal/issues/283
+https://atomgit.com/openeuler/openEuler-portal/issues/295</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -495,7 +496,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -564,7 +565,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-20 07:39:21</v>
+        <v>2026-09-21 07:48:08</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -672,7 +673,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-20 07:39:21</v>
+        <v>2026-09-21 07:48:08</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -780,13 +781,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-20 07:39:21</v>
+        <v>2026-09-21 07:48:08</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -820,7 +821,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -889,7 +890,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-20 07:39:21</v>
+        <v>2026-09-21 07:48:08</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -997,7 +998,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-20 07:39:21</v>
+        <v>2026-09-21 07:48:08</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1105,13 +1106,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-20 07:39:21</v>
+        <v>2026-09-21 07:48:08</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>84</v>
+        <v>67</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1119,8 +1120,7 @@
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://atomgit.com/mindspore/mindspore-portal/issues/186
 https://atomgit.com/mindspore/mindspore-portal/issues/187
-https://atomgit.com/mindspore/mindspore-portal/issues/188
-https://atomgit.com/mindspore/mindspore-portal/issues/234</v>
+https://atomgit.com/mindspore/mindspore-portal/issues/188</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1129,10 +1129,10 @@
         <v>0</v>
       </c>
       <c r="H2">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="I2">
-        <v>59</v>
+        <v>51</v>
       </c>
       <c r="J2">
         <v>0</v>
@@ -1147,7 +1147,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -1216,13 +1216,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-20 07:39:21</v>
+        <v>2026-09-21 07:48:08</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1248,7 +1248,7 @@
         <v>0</v>
       </c>
       <c r="K2">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="L2">
         <v>0</v>
@@ -1326,13 +1326,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-20 07:39:21</v>
+        <v>2026-09-21 07:48:08</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1341,8 +1341,7 @@
         <v xml:space="preserve">https://atomgit.com/hifloat/hifloat-portal/issues/4
 https://atomgit.com/hifloat/hifloat-portal/issues/5
 https://atomgit.com/hifloat/hifloat-portal/issues/6
-https://atomgit.com/hifloat/hifloat-portal/issues/7
-https://atomgit.com/hifloat/hifloat-portal/issues/8</v>
+https://atomgit.com/hifloat/hifloat-portal/issues/7</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1357,7 +1356,7 @@
         <v>39</v>
       </c>
       <c r="J2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K2">
         <v>1</v>
@@ -1369,7 +1368,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O2">
         <v>0</v>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-09-22
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -454,22 +454,21 @@
         <v>tdk-schema-semantic</v>
       </c>
     </row>
-    <row r="2" xml:space="preserve">
+    <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-21 07:48:08</v>
+        <v>2026-09-22 07:16:04</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
-      <c r="E2" t="str" xml:space="preserve">
-        <v xml:space="preserve">https://atomgit.com/openeuler/openEuler-portal/issues/283
-https://atomgit.com/openeuler/openEuler-portal/issues/295</v>
+      <c r="E2" t="str">
+        <v>https://atomgit.com/openeuler/openEuler-portal/issues/283</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -496,7 +495,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -565,7 +564,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-21 07:48:08</v>
+        <v>2026-09-22 07:16:04</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -673,7 +672,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-21 07:48:08</v>
+        <v>2026-09-22 07:16:04</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -781,13 +780,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-21 07:48:08</v>
+        <v>2026-09-22 07:16:04</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -821,7 +820,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -890,7 +889,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-21 07:48:08</v>
+        <v>2026-09-22 07:16:04</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -998,7 +997,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-21 07:48:08</v>
+        <v>2026-09-22 07:16:04</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1106,7 +1105,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-21 07:48:08</v>
+        <v>2026-09-22 07:16:04</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1216,7 +1215,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-21 07:48:08</v>
+        <v>2026-09-22 07:16:04</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1326,13 +1325,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-21 07:48:08</v>
+        <v>2026-09-22 07:16:04</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1341,7 +1340,8 @@
         <v xml:space="preserve">https://atomgit.com/hifloat/hifloat-portal/issues/4
 https://atomgit.com/hifloat/hifloat-portal/issues/5
 https://atomgit.com/hifloat/hifloat-portal/issues/6
-https://atomgit.com/hifloat/hifloat-portal/issues/7</v>
+https://atomgit.com/hifloat/hifloat-portal/issues/7
+https://atomgit.com/hifloat/hifloat-portal/issues/8</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1368,7 +1368,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O2">
         <v>0</v>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-09-23
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,7 +456,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-22 07:16:04</v>
+        <v>2026-09-23 07:13:54</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -564,7 +564,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-22 07:16:04</v>
+        <v>2026-09-23 07:13:54</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -672,7 +672,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-22 07:16:04</v>
+        <v>2026-09-23 07:13:54</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -780,13 +780,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-22 07:16:04</v>
+        <v>2026-09-23 07:13:54</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -820,7 +820,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -889,7 +889,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-22 07:16:04</v>
+        <v>2026-09-23 07:13:54</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -997,7 +997,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-22 07:16:04</v>
+        <v>2026-09-23 07:13:54</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1105,7 +1105,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-22 07:16:04</v>
+        <v>2026-09-23 07:13:54</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1215,13 +1215,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-22 07:16:04</v>
+        <v>2026-09-23 07:13:54</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>186</v>
+        <v>191</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1241,7 +1241,7 @@
         <v>2</v>
       </c>
       <c r="I2">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="J2">
         <v>0</v>
@@ -1325,13 +1325,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-22 07:16:04</v>
+        <v>2026-09-23 07:13:54</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1340,8 +1340,7 @@
         <v xml:space="preserve">https://atomgit.com/hifloat/hifloat-portal/issues/4
 https://atomgit.com/hifloat/hifloat-portal/issues/5
 https://atomgit.com/hifloat/hifloat-portal/issues/6
-https://atomgit.com/hifloat/hifloat-portal/issues/7
-https://atomgit.com/hifloat/hifloat-portal/issues/8</v>
+https://atomgit.com/hifloat/hifloat-portal/issues/7</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1356,7 +1355,7 @@
         <v>39</v>
       </c>
       <c r="J2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K2">
         <v>1</v>
@@ -1368,7 +1367,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O2">
         <v>0</v>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-09-24
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,7 +456,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-23 07:13:54</v>
+        <v>2026-09-24 07:10:04</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -564,7 +564,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-23 07:13:54</v>
+        <v>2026-09-24 07:10:04</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -672,7 +672,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-23 07:13:54</v>
+        <v>2026-09-24 07:10:04</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -780,13 +780,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-23 07:13:54</v>
+        <v>2026-09-24 07:10:04</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -820,7 +820,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -889,7 +889,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-23 07:13:54</v>
+        <v>2026-09-24 07:10:04</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -997,7 +997,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-23 07:13:54</v>
+        <v>2026-09-24 07:10:04</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1105,7 +1105,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-23 07:13:54</v>
+        <v>2026-09-24 07:10:04</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1215,21 +1215,22 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-23 07:13:54</v>
+        <v>2026-09-24 07:10:04</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
       <c r="E2" t="str" xml:space="preserve">
-        <v xml:space="preserve">https://atomgit.com/openUBMC/website/issues/151
+        <v xml:space="preserve">https://gitcode.com/openUBMC/website/issues/151
 https://atomgit.com/openUBMC/website/issues/152
-https://atomgit.com/openUBMC/website/issues/153</v>
+https://atomgit.com/openUBMC/website/issues/153
+https://atomgit.com/openUBMC/website/issues/185</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1241,7 +1242,7 @@
         <v>2</v>
       </c>
       <c r="I2">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="J2">
         <v>0</v>
@@ -1256,7 +1257,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -1325,13 +1326,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-23 07:13:54</v>
+        <v>2026-09-24 07:10:04</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1340,7 +1341,8 @@
         <v xml:space="preserve">https://atomgit.com/hifloat/hifloat-portal/issues/4
 https://atomgit.com/hifloat/hifloat-portal/issues/5
 https://atomgit.com/hifloat/hifloat-portal/issues/6
-https://atomgit.com/hifloat/hifloat-portal/issues/7</v>
+https://atomgit.com/hifloat/hifloat-portal/issues/7
+https://atomgit.com/hifloat/hifloat-portal/issues/8</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1367,7 +1369,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O2">
         <v>0</v>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-09-25
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,20 +456,20 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-24 07:10:04</v>
+        <v>2026-09-25 07:05:04</v>
       </c>
       <c r="B2" t="str">
-        <v>成功</v>
+        <v>失败</v>
       </c>
       <c r="C2">
-        <v>242</v>
+        <v>0</v>
       </c>
       <c r="D2" t="str">
+        <v>spawnSync /bin/sh ETIMEDOUT</v>
+      </c>
+      <c r="E2" t="str">
         <v/>
       </c>
-      <c r="E2" t="str">
-        <v>https://atomgit.com/openeuler/openEuler-portal/issues/283</v>
-      </c>
       <c r="F2">
         <v>0</v>
       </c>
@@ -480,7 +480,7 @@
         <v>0</v>
       </c>
       <c r="I2">
-        <v>242</v>
+        <v>0</v>
       </c>
       <c r="J2">
         <v>0</v>
@@ -564,7 +564,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-24 07:10:04</v>
+        <v>2026-09-25 07:05:04</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -672,7 +672,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-24 07:10:04</v>
+        <v>2026-09-25 07:05:04</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -780,20 +780,20 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-24 07:10:04</v>
+        <v>2026-09-25 07:05:04</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
       <c r="E2" t="str" xml:space="preserve">
-        <v xml:space="preserve">https://atomgit.com/opengauss/website/issues/367
-https://atomgit.com/opengauss/website/issues/360</v>
+        <v xml:space="preserve">https://gitcode.com/opengauss/website/issues/367
+https://gitcode.com/opengauss/website/issues/360</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -820,7 +820,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -889,7 +889,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-24 07:10:04</v>
+        <v>2026-09-25 07:05:04</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -997,7 +997,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-24 07:10:04</v>
+        <v>2026-09-25 07:05:04</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1105,7 +1105,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-24 07:10:04</v>
+        <v>2026-09-25 07:05:04</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1118,8 +1118,8 @@
       </c>
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://atomgit.com/mindspore/mindspore-portal/issues/186
-https://atomgit.com/mindspore/mindspore-portal/issues/187
-https://atomgit.com/mindspore/mindspore-portal/issues/188</v>
+https://gitcode.com/mindspore/mindspore-portal/issues/187
+https://gitcode.com/mindspore/mindspore-portal/issues/188</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1215,7 +1215,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-24 07:10:04</v>
+        <v>2026-09-25 07:05:04</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1228,7 +1228,7 @@
       </c>
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://gitcode.com/openUBMC/website/issues/151
-https://atomgit.com/openUBMC/website/issues/152
+https://gitcode.com/openUBMC/website/issues/152
 https://atomgit.com/openUBMC/website/issues/153
 https://atomgit.com/openUBMC/website/issues/185</v>
       </c>
@@ -1326,23 +1326,23 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-24 07:10:04</v>
+        <v>2026-09-25 07:05:04</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
       <c r="E2" t="str" xml:space="preserve">
-        <v xml:space="preserve">https://atomgit.com/hifloat/hifloat-portal/issues/4
-https://atomgit.com/hifloat/hifloat-portal/issues/5
+        <v xml:space="preserve">https://gitcode.com/hifloat/hifloat-portal/issues/4
+https://gitcode.com/hifloat/hifloat-portal/issues/5
 https://atomgit.com/hifloat/hifloat-portal/issues/6
-https://atomgit.com/hifloat/hifloat-portal/issues/7
-https://atomgit.com/hifloat/hifloat-portal/issues/8</v>
+https://gitcode.com/hifloat/hifloat-portal/issues/7
+https://gitcode.com/hifloat/hifloat-portal/issues/8</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1369,7 +1369,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O2">
         <v>0</v>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-09-26
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,19 +456,19 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-25 07:05:04</v>
+        <v>2026-09-26 07:07:30</v>
       </c>
       <c r="B2" t="str">
-        <v>失败</v>
+        <v>成功</v>
       </c>
       <c r="C2">
-        <v>0</v>
+        <v>244</v>
       </c>
       <c r="D2" t="str">
-        <v>spawnSync /bin/sh ETIMEDOUT</v>
+        <v/>
       </c>
       <c r="E2" t="str">
-        <v/>
+        <v>https://atomgit.com/openeuler/openEuler-portal/issues/283</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -480,7 +480,7 @@
         <v>0</v>
       </c>
       <c r="I2">
-        <v>0</v>
+        <v>244</v>
       </c>
       <c r="J2">
         <v>0</v>
@@ -564,7 +564,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-25 07:05:04</v>
+        <v>2026-09-26 07:07:30</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -672,7 +672,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-25 07:05:04</v>
+        <v>2026-09-26 07:07:30</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -780,20 +780,20 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-25 07:05:04</v>
+        <v>2026-09-26 07:07:30</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://gitcode.com/opengauss/website/issues/367
-https://gitcode.com/opengauss/website/issues/360</v>
+https://atomgit.com/opengauss/website/issues/360</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -820,7 +820,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -889,7 +889,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-25 07:05:04</v>
+        <v>2026-09-26 07:07:30</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -997,7 +997,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-25 07:05:04</v>
+        <v>2026-09-26 07:07:30</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1105,7 +1105,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-25 07:05:04</v>
+        <v>2026-09-26 07:07:30</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1117,9 +1117,9 @@
         <v/>
       </c>
       <c r="E2" t="str" xml:space="preserve">
-        <v xml:space="preserve">https://atomgit.com/mindspore/mindspore-portal/issues/186
+        <v xml:space="preserve">https://gitcode.com/mindspore/mindspore-portal/issues/186
 https://gitcode.com/mindspore/mindspore-portal/issues/187
-https://gitcode.com/mindspore/mindspore-portal/issues/188</v>
+https://atomgit.com/mindspore/mindspore-portal/issues/188</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1215,22 +1215,21 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-25 07:05:04</v>
+        <v>2026-09-26 07:07:30</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
       <c r="E2" t="str" xml:space="preserve">
-        <v xml:space="preserve">https://gitcode.com/openUBMC/website/issues/151
+        <v xml:space="preserve">https://atomgit.com/openUBMC/website/issues/151
 https://gitcode.com/openUBMC/website/issues/152
-https://atomgit.com/openUBMC/website/issues/153
-https://atomgit.com/openUBMC/website/issues/185</v>
+https://atomgit.com/openUBMC/website/issues/153</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1257,7 +1256,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -1326,22 +1325,22 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-25 07:05:04</v>
+        <v>2026-09-26 07:07:30</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
       <c r="E2" t="str" xml:space="preserve">
-        <v xml:space="preserve">https://gitcode.com/hifloat/hifloat-portal/issues/4
-https://gitcode.com/hifloat/hifloat-portal/issues/5
+        <v xml:space="preserve">https://atomgit.com/hifloat/hifloat-portal/issues/4
+https://atomgit.com/hifloat/hifloat-portal/issues/5
 https://atomgit.com/hifloat/hifloat-portal/issues/6
-https://gitcode.com/hifloat/hifloat-portal/issues/7
+https://atomgit.com/hifloat/hifloat-portal/issues/7
 https://gitcode.com/hifloat/hifloat-portal/issues/8</v>
       </c>
       <c r="F2">
@@ -1369,7 +1368,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O2">
         <v>0</v>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-09-27
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,7 +456,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-26 07:07:30</v>
+        <v>2026-09-27 07:31:49</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -468,7 +468,7 @@
         <v/>
       </c>
       <c r="E2" t="str">
-        <v>https://atomgit.com/openeuler/openEuler-portal/issues/283</v>
+        <v>https://gitcode.com/openeuler/openEuler-portal/issues/283</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -564,7 +564,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-26 07:07:30</v>
+        <v>2026-09-27 07:31:49</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -672,7 +672,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-26 07:07:30</v>
+        <v>2026-09-27 07:31:49</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -780,20 +780,20 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-26 07:07:30</v>
+        <v>2026-09-27 07:31:49</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
       <c r="E2" t="str" xml:space="preserve">
-        <v xml:space="preserve">https://gitcode.com/opengauss/website/issues/367
-https://atomgit.com/opengauss/website/issues/360</v>
+        <v xml:space="preserve">https://atomgit.com/opengauss/website/issues/367
+https://gitcode.com/opengauss/website/issues/360</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -820,7 +820,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -889,7 +889,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-26 07:07:30</v>
+        <v>2026-09-27 07:31:49</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -997,7 +997,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-26 07:07:30</v>
+        <v>2026-09-27 07:31:49</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1105,7 +1105,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-26 07:07:30</v>
+        <v>2026-09-27 07:31:49</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1119,7 +1119,7 @@
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://gitcode.com/mindspore/mindspore-portal/issues/186
 https://gitcode.com/mindspore/mindspore-portal/issues/187
-https://atomgit.com/mindspore/mindspore-portal/issues/188</v>
+https://gitcode.com/mindspore/mindspore-portal/issues/188</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1215,7 +1215,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-26 07:07:30</v>
+        <v>2026-09-27 07:31:49</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1227,9 +1227,9 @@
         <v/>
       </c>
       <c r="E2" t="str" xml:space="preserve">
-        <v xml:space="preserve">https://atomgit.com/openUBMC/website/issues/151
+        <v xml:space="preserve">https://gitcode.com/openUBMC/website/issues/151
 https://gitcode.com/openUBMC/website/issues/152
-https://atomgit.com/openUBMC/website/issues/153</v>
+https://gitcode.com/openUBMC/website/issues/153</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1325,7 +1325,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-26 07:07:30</v>
+        <v>2026-09-27 07:31:49</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1356,7 +1356,7 @@
         <v>39</v>
       </c>
       <c r="J2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K2">
         <v>1</v>
@@ -1368,7 +1368,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O2">
         <v>0</v>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-09-28
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,7 +456,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-27 07:31:49</v>
+        <v>2026-09-28 08:21:30</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -468,7 +468,7 @@
         <v/>
       </c>
       <c r="E2" t="str">
-        <v>https://gitcode.com/openeuler/openEuler-portal/issues/283</v>
+        <v>https://atomgit.com/openeuler/openEuler-portal/issues/283</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -564,7 +564,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-27 07:31:49</v>
+        <v>2026-09-28 08:21:30</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -672,7 +672,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-27 07:31:49</v>
+        <v>2026-09-28 08:21:30</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -780,20 +780,20 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-27 07:31:49</v>
+        <v>2026-09-28 08:21:30</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://atomgit.com/opengauss/website/issues/367
-https://gitcode.com/opengauss/website/issues/360</v>
+https://atomgit.com/opengauss/website/issues/360</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -820,7 +820,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -889,7 +889,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-27 07:31:49</v>
+        <v>2026-09-28 08:21:30</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -997,7 +997,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-27 07:31:49</v>
+        <v>2026-09-28 08:21:30</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1105,7 +1105,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-27 07:31:49</v>
+        <v>2026-09-28 08:21:30</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1118,8 +1118,8 @@
       </c>
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://gitcode.com/mindspore/mindspore-portal/issues/186
-https://gitcode.com/mindspore/mindspore-portal/issues/187
-https://gitcode.com/mindspore/mindspore-portal/issues/188</v>
+https://atomgit.com/mindspore/mindspore-portal/issues/187
+https://atomgit.com/mindspore/mindspore-portal/issues/188</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1215,7 +1215,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-27 07:31:49</v>
+        <v>2026-09-28 08:21:30</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1227,8 +1227,8 @@
         <v/>
       </c>
       <c r="E2" t="str" xml:space="preserve">
-        <v xml:space="preserve">https://gitcode.com/openUBMC/website/issues/151
-https://gitcode.com/openUBMC/website/issues/152
+        <v xml:space="preserve">https://atomgit.com/openUBMC/website/issues/151
+https://atomgit.com/openUBMC/website/issues/152
 https://gitcode.com/openUBMC/website/issues/153</v>
       </c>
       <c r="F2">
@@ -1325,23 +1325,22 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-27 07:31:49</v>
+        <v>2026-09-28 08:21:30</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
       <c r="E2" t="str" xml:space="preserve">
-        <v xml:space="preserve">https://atomgit.com/hifloat/hifloat-portal/issues/4
+        <v xml:space="preserve">https://gitcode.com/hifloat/hifloat-portal/issues/4
 https://atomgit.com/hifloat/hifloat-portal/issues/5
 https://atomgit.com/hifloat/hifloat-portal/issues/6
-https://atomgit.com/hifloat/hifloat-portal/issues/7
-https://gitcode.com/hifloat/hifloat-portal/issues/8</v>
+https://gitcode.com/hifloat/hifloat-portal/issues/7</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1350,10 +1349,10 @@
         <v>0</v>
       </c>
       <c r="H2">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="I2">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="J2">
         <v>2</v>
@@ -1368,7 +1367,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O2">
         <v>0</v>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-09-29
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,7 +456,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-28 08:21:30</v>
+        <v>2026-09-29 07:53:33</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -564,7 +564,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-28 08:21:30</v>
+        <v>2026-09-29 07:53:33</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -672,7 +672,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-28 08:21:30</v>
+        <v>2026-09-29 07:53:33</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -780,20 +780,20 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-28 08:21:30</v>
+        <v>2026-09-29 07:53:33</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://atomgit.com/opengauss/website/issues/367
-https://atomgit.com/opengauss/website/issues/360</v>
+https://gitcode.com/opengauss/website/issues/360</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -820,7 +820,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -889,7 +889,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-28 08:21:30</v>
+        <v>2026-09-29 07:53:33</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -997,7 +997,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-28 08:21:30</v>
+        <v>2026-09-29 07:53:33</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1105,7 +1105,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-28 08:21:30</v>
+        <v>2026-09-29 07:53:33</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1119,7 +1119,7 @@
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://gitcode.com/mindspore/mindspore-portal/issues/186
 https://atomgit.com/mindspore/mindspore-portal/issues/187
-https://atomgit.com/mindspore/mindspore-portal/issues/188</v>
+https://gitcode.com/mindspore/mindspore-portal/issues/188</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1215,7 +1215,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-28 08:21:30</v>
+        <v>2026-09-29 07:53:33</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1227,9 +1227,9 @@
         <v/>
       </c>
       <c r="E2" t="str" xml:space="preserve">
-        <v xml:space="preserve">https://atomgit.com/openUBMC/website/issues/151
+        <v xml:space="preserve">https://gitcode.com/openUBMC/website/issues/151
 https://atomgit.com/openUBMC/website/issues/152
-https://gitcode.com/openUBMC/website/issues/153</v>
+https://atomgit.com/openUBMC/website/issues/153</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1325,22 +1325,22 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-28 08:21:30</v>
+        <v>2026-09-29 07:53:33</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
       <c r="E2" t="str" xml:space="preserve">
-        <v xml:space="preserve">https://gitcode.com/hifloat/hifloat-portal/issues/4
-https://atomgit.com/hifloat/hifloat-portal/issues/5
-https://atomgit.com/hifloat/hifloat-portal/issues/6
-https://gitcode.com/hifloat/hifloat-portal/issues/7</v>
+        <v xml:space="preserve">https://atomgit.com/hifloat/hifloat-portal/issues/4
+https://gitcode.com/hifloat/hifloat-portal/issues/5
+https://atomgit.com/hifloat/hifloat-portal/issues/7
+https://gitcode.com/hifloat/hifloat-portal/issues/8</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1355,7 +1355,7 @@
         <v>41</v>
       </c>
       <c r="J2">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K2">
         <v>1</v>
@@ -1367,7 +1367,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O2">
         <v>0</v>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-09-30
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,7 +456,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-29 07:53:33</v>
+        <v>2026-09-30 08:13:26</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -468,7 +468,7 @@
         <v/>
       </c>
       <c r="E2" t="str">
-        <v>https://atomgit.com/openeuler/openEuler-portal/issues/283</v>
+        <v>https://gitcode.com/openeuler/openEuler-portal/issues/283</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -564,7 +564,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-29 07:53:33</v>
+        <v>2026-09-30 08:13:26</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -672,7 +672,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-29 07:53:33</v>
+        <v>2026-09-30 08:13:26</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -780,20 +780,21 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-29 07:53:33</v>
+        <v>2026-09-30 08:13:26</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://atomgit.com/opengauss/website/issues/367
-https://gitcode.com/opengauss/website/issues/360</v>
+https://gitcode.com/opengauss/website/issues/360
+https://atomgit.com/opengauss/website/issues/399</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -817,7 +818,7 @@
         <v>0</v>
       </c>
       <c r="M2">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="N2">
         <v>4</v>
@@ -889,7 +890,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-29 07:53:33</v>
+        <v>2026-09-30 08:13:26</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -997,7 +998,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-29 07:53:33</v>
+        <v>2026-09-30 08:13:26</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1105,7 +1106,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-29 07:53:33</v>
+        <v>2026-09-30 08:13:26</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1119,7 +1120,7 @@
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://gitcode.com/mindspore/mindspore-portal/issues/186
 https://atomgit.com/mindspore/mindspore-portal/issues/187
-https://gitcode.com/mindspore/mindspore-portal/issues/188</v>
+https://atomgit.com/mindspore/mindspore-portal/issues/188</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1215,21 +1216,21 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-29 07:53:33</v>
+        <v>2026-09-30 08:13:26</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>186</v>
+        <v>192</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
       <c r="E2" t="str" xml:space="preserve">
-        <v xml:space="preserve">https://gitcode.com/openUBMC/website/issues/151
-https://atomgit.com/openUBMC/website/issues/152
-https://atomgit.com/openUBMC/website/issues/153</v>
+        <v xml:space="preserve">https://atomgit.com/openUBMC/website/issues/151
+https://gitcode.com/openUBMC/website/issues/152
+https://gitcode.com/openUBMC/website/issues/153</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1241,13 +1242,13 @@
         <v>2</v>
       </c>
       <c r="I2">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="L2">
         <v>0</v>
@@ -1325,7 +1326,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-29 07:53:33</v>
+        <v>2026-09-30 08:13:26</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1337,10 +1338,10 @@
         <v/>
       </c>
       <c r="E2" t="str" xml:space="preserve">
-        <v xml:space="preserve">https://atomgit.com/hifloat/hifloat-portal/issues/4
+        <v xml:space="preserve">https://gitcode.com/hifloat/hifloat-portal/issues/4
 https://gitcode.com/hifloat/hifloat-portal/issues/5
-https://atomgit.com/hifloat/hifloat-portal/issues/7
-https://gitcode.com/hifloat/hifloat-portal/issues/8</v>
+https://gitcode.com/hifloat/hifloat-portal/issues/6
+https://atomgit.com/hifloat/hifloat-portal/issues/7</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1355,7 +1356,7 @@
         <v>41</v>
       </c>
       <c r="J2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K2">
         <v>1</v>
@@ -1367,7 +1368,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O2">
         <v>0</v>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-10-01
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,13 +456,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-30 08:13:26</v>
+        <v>2026-10-01 08:28:15</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>244</v>
+        <v>4</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -480,7 +480,7 @@
         <v>0</v>
       </c>
       <c r="I2">
-        <v>244</v>
+        <v>4</v>
       </c>
       <c r="J2">
         <v>0</v>
@@ -564,7 +564,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-30 08:13:26</v>
+        <v>2026-10-01 08:28:15</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -672,7 +672,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-30 08:13:26</v>
+        <v>2026-10-01 08:28:15</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -780,21 +780,21 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-30 08:13:26</v>
+        <v>2026-10-01 08:28:15</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
       <c r="E2" t="str" xml:space="preserve">
-        <v xml:space="preserve">https://atomgit.com/opengauss/website/issues/367
-https://gitcode.com/opengauss/website/issues/360
-https://atomgit.com/opengauss/website/issues/399</v>
+        <v xml:space="preserve">https://atomgit.com/opengauss/website/issues/404
+https://atomgit.com/opengauss/website/issues/367
+https://gitcode.com/opengauss/website/issues/360</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -806,19 +806,19 @@
         <v>0</v>
       </c>
       <c r="I2">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="L2">
         <v>0</v>
       </c>
       <c r="M2">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="N2">
         <v>4</v>
@@ -890,7 +890,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-30 08:13:26</v>
+        <v>2026-10-01 08:28:15</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -998,7 +998,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-30 08:13:26</v>
+        <v>2026-10-01 08:28:15</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1106,20 +1106,20 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-30 08:13:26</v>
+        <v>2026-10-01 08:28:15</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
       <c r="E2" t="str" xml:space="preserve">
-        <v xml:space="preserve">https://gitcode.com/mindspore/mindspore-portal/issues/186
-https://atomgit.com/mindspore/mindspore-portal/issues/187
+        <v xml:space="preserve">https://atomgit.com/mindspore/mindspore-portal/issues/187
+https://atomgit.com/mindspore/mindspore-portal/issues/186
 https://atomgit.com/mindspore/mindspore-portal/issues/188</v>
       </c>
       <c r="F2">
@@ -1129,7 +1129,7 @@
         <v>0</v>
       </c>
       <c r="H2">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="I2">
         <v>51</v>
@@ -1216,7 +1216,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-30 08:13:26</v>
+        <v>2026-10-01 08:28:15</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1228,8 +1228,8 @@
         <v/>
       </c>
       <c r="E2" t="str" xml:space="preserve">
-        <v xml:space="preserve">https://atomgit.com/openUBMC/website/issues/151
-https://gitcode.com/openUBMC/website/issues/152
+        <v xml:space="preserve">https://gitcode.com/openUBMC/website/issues/151
+https://atomgit.com/openUBMC/website/issues/152
 https://gitcode.com/openUBMC/website/issues/153</v>
       </c>
       <c r="F2">
@@ -1326,22 +1326,21 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-09-30 08:13:26</v>
+        <v>2026-10-01 08:28:15</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
       <c r="E2" t="str" xml:space="preserve">
-        <v xml:space="preserve">https://gitcode.com/hifloat/hifloat-portal/issues/4
+        <v xml:space="preserve">https://atomgit.com/hifloat/hifloat-portal/issues/4
 https://gitcode.com/hifloat/hifloat-portal/issues/5
-https://gitcode.com/hifloat/hifloat-portal/issues/6
-https://atomgit.com/hifloat/hifloat-portal/issues/7</v>
+https://gitcode.com/hifloat/hifloat-portal/issues/7</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1356,7 +1355,7 @@
         <v>41</v>
       </c>
       <c r="J2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K2">
         <v>1</v>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-10-02
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,7 +456,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-01 08:28:15</v>
+        <v>2026-10-02 07:59:50</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -564,7 +564,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-01 08:28:15</v>
+        <v>2026-10-02 07:59:50</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -672,7 +672,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-01 08:28:15</v>
+        <v>2026-10-02 07:59:50</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -780,13 +780,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-01 08:28:15</v>
+        <v>2026-10-02 07:59:50</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -794,7 +794,7 @@
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://atomgit.com/opengauss/website/issues/404
 https://atomgit.com/opengauss/website/issues/367
-https://gitcode.com/opengauss/website/issues/360</v>
+https://atomgit.com/opengauss/website/issues/360</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -821,7 +821,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -890,7 +890,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-01 08:28:15</v>
+        <v>2026-10-02 07:59:50</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -998,7 +998,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-01 08:28:15</v>
+        <v>2026-10-02 07:59:50</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1106,7 +1106,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-01 08:28:15</v>
+        <v>2026-10-02 07:59:50</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1120,7 +1120,7 @@
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://atomgit.com/mindspore/mindspore-portal/issues/187
 https://atomgit.com/mindspore/mindspore-portal/issues/186
-https://atomgit.com/mindspore/mindspore-portal/issues/188</v>
+https://gitcode.com/mindspore/mindspore-portal/issues/188</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1216,7 +1216,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-01 08:28:15</v>
+        <v>2026-10-02 07:59:50</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1229,7 +1229,7 @@
       </c>
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://gitcode.com/openUBMC/website/issues/151
-https://atomgit.com/openUBMC/website/issues/152
+https://gitcode.com/openUBMC/website/issues/152
 https://gitcode.com/openUBMC/website/issues/153</v>
       </c>
       <c r="F2">
@@ -1326,21 +1326,22 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-01 08:28:15</v>
+        <v>2026-10-02 07:59:50</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
       <c r="E2" t="str" xml:space="preserve">
-        <v xml:space="preserve">https://atomgit.com/hifloat/hifloat-portal/issues/4
+        <v xml:space="preserve">https://gitcode.com/hifloat/hifloat-portal/issues/4
 https://gitcode.com/hifloat/hifloat-portal/issues/5
-https://gitcode.com/hifloat/hifloat-portal/issues/7</v>
+https://atomgit.com/hifloat/hifloat-portal/issues/7
+https://atomgit.com/hifloat/hifloat-portal/issues/8</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1367,7 +1368,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O2">
         <v>0</v>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-10-03
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -454,21 +454,22 @@
         <v>tdk-schema-semantic</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-02 07:59:50</v>
+        <v>2026-10-03 07:29:35</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
-      <c r="E2" t="str">
-        <v>https://gitcode.com/openeuler/openEuler-portal/issues/283</v>
+      <c r="E2" t="str" xml:space="preserve">
+        <v xml:space="preserve">https://gitcode.com/openeuler/openEuler-portal/issues/283
+https://atomgit.com/openeuler/openEuler-portal/issues/324</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -495,7 +496,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -564,7 +565,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-02 07:59:50</v>
+        <v>2026-10-03 07:29:35</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -672,7 +673,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-02 07:59:50</v>
+        <v>2026-10-03 07:29:35</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -780,20 +781,20 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-02 07:59:50</v>
+        <v>2026-10-03 07:29:35</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
       <c r="E2" t="str" xml:space="preserve">
-        <v xml:space="preserve">https://atomgit.com/opengauss/website/issues/404
-https://atomgit.com/opengauss/website/issues/367
+        <v xml:space="preserve">https://gitcode.com/opengauss/website/issues/404
+https://gitcode.com/opengauss/website/issues/367
 https://atomgit.com/opengauss/website/issues/360</v>
       </c>
       <c r="F2">
@@ -821,7 +822,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -890,7 +891,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-02 07:59:50</v>
+        <v>2026-10-03 07:29:35</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -998,7 +999,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-02 07:59:50</v>
+        <v>2026-10-03 07:29:35</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1106,7 +1107,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-02 07:59:50</v>
+        <v>2026-10-03 07:29:35</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1118,7 +1119,7 @@
         <v/>
       </c>
       <c r="E2" t="str" xml:space="preserve">
-        <v xml:space="preserve">https://atomgit.com/mindspore/mindspore-portal/issues/187
+        <v xml:space="preserve">https://gitcode.com/mindspore/mindspore-portal/issues/187
 https://atomgit.com/mindspore/mindspore-portal/issues/186
 https://gitcode.com/mindspore/mindspore-portal/issues/188</v>
       </c>
@@ -1216,7 +1217,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-02 07:59:50</v>
+        <v>2026-10-03 07:29:35</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1229,8 +1230,8 @@
       </c>
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://gitcode.com/openUBMC/website/issues/151
-https://gitcode.com/openUBMC/website/issues/152
-https://gitcode.com/openUBMC/website/issues/153</v>
+https://atomgit.com/openUBMC/website/issues/152
+https://atomgit.com/openUBMC/website/issues/153</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1326,13 +1327,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-02 07:59:50</v>
+        <v>2026-10-03 07:29:35</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1340,7 +1341,8 @@
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://gitcode.com/hifloat/hifloat-portal/issues/4
 https://gitcode.com/hifloat/hifloat-portal/issues/5
-https://atomgit.com/hifloat/hifloat-portal/issues/7
+https://atomgit.com/hifloat/hifloat-portal/issues/6
+https://gitcode.com/hifloat/hifloat-portal/issues/7
 https://atomgit.com/hifloat/hifloat-portal/issues/8</v>
       </c>
       <c r="F2">
@@ -1356,7 +1358,7 @@
         <v>41</v>
       </c>
       <c r="J2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K2">
         <v>1</v>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-10-04
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -454,22 +454,21 @@
         <v>tdk-schema-semantic</v>
       </c>
     </row>
-    <row r="2" xml:space="preserve">
+    <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-03 07:29:35</v>
+        <v>2026-10-04 07:44:55</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
-      <c r="E2" t="str" xml:space="preserve">
-        <v xml:space="preserve">https://gitcode.com/openeuler/openEuler-portal/issues/283
-https://atomgit.com/openeuler/openEuler-portal/issues/324</v>
+      <c r="E2" t="str">
+        <v>https://gitcode.com/openeuler/openEuler-portal/issues/283</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -496,7 +495,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -565,7 +564,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-03 07:29:35</v>
+        <v>2026-10-04 07:44:55</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -673,7 +672,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-03 07:29:35</v>
+        <v>2026-10-04 07:44:55</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -781,19 +780,19 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-03 07:29:35</v>
+        <v>2026-10-04 07:44:55</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
       <c r="E2" t="str" xml:space="preserve">
-        <v xml:space="preserve">https://gitcode.com/opengauss/website/issues/404
+        <v xml:space="preserve">https://atomgit.com/opengauss/website/issues/404
 https://gitcode.com/opengauss/website/issues/367
 https://atomgit.com/opengauss/website/issues/360</v>
       </c>
@@ -822,7 +821,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -891,7 +890,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-03 07:29:35</v>
+        <v>2026-10-04 07:44:55</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -999,7 +998,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-03 07:29:35</v>
+        <v>2026-10-04 07:44:55</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1107,7 +1106,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-03 07:29:35</v>
+        <v>2026-10-04 07:44:55</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1121,7 +1120,7 @@
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://gitcode.com/mindspore/mindspore-portal/issues/187
 https://atomgit.com/mindspore/mindspore-portal/issues/186
-https://gitcode.com/mindspore/mindspore-portal/issues/188</v>
+https://atomgit.com/mindspore/mindspore-portal/issues/188</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1217,7 +1216,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-03 07:29:35</v>
+        <v>2026-10-04 07:44:55</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1231,7 +1230,7 @@
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://gitcode.com/openUBMC/website/issues/151
 https://atomgit.com/openUBMC/website/issues/152
-https://atomgit.com/openUBMC/website/issues/153</v>
+https://gitcode.com/openUBMC/website/issues/153</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1327,13 +1326,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-03 07:29:35</v>
+        <v>2026-10-04 07:44:55</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1341,8 +1340,8 @@
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://gitcode.com/hifloat/hifloat-portal/issues/4
 https://gitcode.com/hifloat/hifloat-portal/issues/5
-https://atomgit.com/hifloat/hifloat-portal/issues/6
-https://gitcode.com/hifloat/hifloat-portal/issues/7
+https://gitcode.com/hifloat/hifloat-portal/issues/6
+https://atomgit.com/hifloat/hifloat-portal/issues/7
 https://atomgit.com/hifloat/hifloat-portal/issues/8</v>
       </c>
       <c r="F2">
@@ -1358,7 +1357,7 @@
         <v>41</v>
       </c>
       <c r="J2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K2">
         <v>1</v>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-10-05
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,7 +456,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-04 07:44:55</v>
+        <v>2026-10-05 08:08:42</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -564,7 +564,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-04 07:44:55</v>
+        <v>2026-10-05 08:08:42</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -672,7 +672,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-04 07:44:55</v>
+        <v>2026-10-05 08:08:42</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -780,20 +780,20 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-04 07:44:55</v>
+        <v>2026-10-05 08:08:42</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
       <c r="E2" t="str" xml:space="preserve">
-        <v xml:space="preserve">https://atomgit.com/opengauss/website/issues/404
-https://gitcode.com/opengauss/website/issues/367
+        <v xml:space="preserve">https://gitcode.com/opengauss/website/issues/404
+https://atomgit.com/opengauss/website/issues/367
 https://atomgit.com/opengauss/website/issues/360</v>
       </c>
       <c r="F2">
@@ -821,7 +821,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -890,7 +890,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-04 07:44:55</v>
+        <v>2026-10-05 08:08:42</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -998,7 +998,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-04 07:44:55</v>
+        <v>2026-10-05 08:08:42</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1106,7 +1106,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-04 07:44:55</v>
+        <v>2026-10-05 08:08:42</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1119,8 +1119,8 @@
       </c>
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://gitcode.com/mindspore/mindspore-portal/issues/187
-https://atomgit.com/mindspore/mindspore-portal/issues/186
-https://atomgit.com/mindspore/mindspore-portal/issues/188</v>
+https://gitcode.com/mindspore/mindspore-portal/issues/186
+https://gitcode.com/mindspore/mindspore-portal/issues/188</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1216,7 +1216,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-04 07:44:55</v>
+        <v>2026-10-05 08:08:42</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1229,7 +1229,7 @@
       </c>
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://gitcode.com/openUBMC/website/issues/151
-https://atomgit.com/openUBMC/website/issues/152
+https://gitcode.com/openUBMC/website/issues/152
 https://gitcode.com/openUBMC/website/issues/153</v>
       </c>
       <c r="F2">
@@ -1326,23 +1326,22 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-04 07:44:55</v>
+        <v>2026-10-05 08:08:42</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
       <c r="E2" t="str" xml:space="preserve">
-        <v xml:space="preserve">https://gitcode.com/hifloat/hifloat-portal/issues/4
+        <v xml:space="preserve">https://atomgit.com/hifloat/hifloat-portal/issues/4
 https://gitcode.com/hifloat/hifloat-portal/issues/5
 https://gitcode.com/hifloat/hifloat-portal/issues/6
-https://atomgit.com/hifloat/hifloat-portal/issues/7
-https://atomgit.com/hifloat/hifloat-portal/issues/8</v>
+https://atomgit.com/hifloat/hifloat-portal/issues/7</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1357,7 +1356,7 @@
         <v>41</v>
       </c>
       <c r="J2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K2">
         <v>1</v>
@@ -1369,7 +1368,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O2">
         <v>0</v>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-10-06
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,7 +456,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-05 08:08:42</v>
+        <v>2026-10-06 08:42:32</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -564,7 +564,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-05 08:08:42</v>
+        <v>2026-10-06 08:42:32</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -672,7 +672,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-05 08:08:42</v>
+        <v>2026-10-06 08:42:32</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -780,21 +780,21 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-05 08:08:42</v>
+        <v>2026-10-06 08:42:32</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
       <c r="E2" t="str" xml:space="preserve">
-        <v xml:space="preserve">https://gitcode.com/opengauss/website/issues/404
-https://atomgit.com/opengauss/website/issues/367
-https://atomgit.com/opengauss/website/issues/360</v>
+        <v xml:space="preserve">https://atomgit.com/opengauss/website/issues/404
+https://gitcode.com/opengauss/website/issues/367
+https://gitcode.com/opengauss/website/issues/360</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -821,7 +821,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -890,7 +890,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-05 08:08:42</v>
+        <v>2026-10-06 08:42:32</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -998,7 +998,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-05 08:08:42</v>
+        <v>2026-10-06 08:42:32</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1106,13 +1106,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-05 08:08:42</v>
+        <v>2026-10-06 08:42:32</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>60</v>
+        <v>76</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1120,7 +1120,7 @@
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://gitcode.com/mindspore/mindspore-portal/issues/187
 https://gitcode.com/mindspore/mindspore-portal/issues/186
-https://gitcode.com/mindspore/mindspore-portal/issues/188</v>
+https://atomgit.com/mindspore/mindspore-portal/issues/188</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1129,7 +1129,7 @@
         <v>0</v>
       </c>
       <c r="H2">
-        <v>5</v>
+        <v>21</v>
       </c>
       <c r="I2">
         <v>51</v>
@@ -1216,7 +1216,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-05 08:08:42</v>
+        <v>2026-10-06 08:42:32</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1228,8 +1228,8 @@
         <v/>
       </c>
       <c r="E2" t="str" xml:space="preserve">
-        <v xml:space="preserve">https://gitcode.com/openUBMC/website/issues/151
-https://gitcode.com/openUBMC/website/issues/152
+        <v xml:space="preserve">https://atomgit.com/openUBMC/website/issues/151
+https://atomgit.com/openUBMC/website/issues/152
 https://gitcode.com/openUBMC/website/issues/153</v>
       </c>
       <c r="F2">
@@ -1326,7 +1326,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-05 08:08:42</v>
+        <v>2026-10-06 08:42:32</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1338,10 +1338,10 @@
         <v/>
       </c>
       <c r="E2" t="str" xml:space="preserve">
-        <v xml:space="preserve">https://atomgit.com/hifloat/hifloat-portal/issues/4
+        <v xml:space="preserve">https://gitcode.com/hifloat/hifloat-portal/issues/4
 https://gitcode.com/hifloat/hifloat-portal/issues/5
-https://gitcode.com/hifloat/hifloat-portal/issues/6
-https://atomgit.com/hifloat/hifloat-portal/issues/7</v>
+https://atomgit.com/hifloat/hifloat-portal/issues/7
+https://atomgit.com/hifloat/hifloat-portal/issues/8</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1356,7 +1356,7 @@
         <v>41</v>
       </c>
       <c r="J2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K2">
         <v>1</v>
@@ -1368,7 +1368,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O2">
         <v>0</v>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-10-07
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,7 +456,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-06 08:42:32</v>
+        <v>2026-10-07 08:06:59</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -564,7 +564,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-06 08:42:32</v>
+        <v>2026-10-07 08:06:59</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -672,7 +672,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-06 08:42:32</v>
+        <v>2026-10-07 08:06:59</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -780,7 +780,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-06 08:42:32</v>
+        <v>2026-10-07 08:06:59</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -792,8 +792,8 @@
         <v/>
       </c>
       <c r="E2" t="str" xml:space="preserve">
-        <v xml:space="preserve">https://atomgit.com/opengauss/website/issues/404
-https://gitcode.com/opengauss/website/issues/367
+        <v xml:space="preserve">https://gitcode.com/opengauss/website/issues/404
+https://atomgit.com/opengauss/website/issues/367
 https://gitcode.com/opengauss/website/issues/360</v>
       </c>
       <c r="F2">
@@ -890,7 +890,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-06 08:42:32</v>
+        <v>2026-10-07 08:06:59</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -998,7 +998,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-06 08:42:32</v>
+        <v>2026-10-07 08:06:59</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1106,21 +1106,21 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-06 08:42:32</v>
+        <v>2026-10-07 08:06:59</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>76</v>
+        <v>60</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
       <c r="E2" t="str" xml:space="preserve">
-        <v xml:space="preserve">https://gitcode.com/mindspore/mindspore-portal/issues/187
+        <v xml:space="preserve">https://atomgit.com/mindspore/mindspore-portal/issues/187
 https://gitcode.com/mindspore/mindspore-portal/issues/186
-https://atomgit.com/mindspore/mindspore-portal/issues/188</v>
+https://gitcode.com/mindspore/mindspore-portal/issues/188</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1129,7 +1129,7 @@
         <v>0</v>
       </c>
       <c r="H2">
-        <v>21</v>
+        <v>5</v>
       </c>
       <c r="I2">
         <v>51</v>
@@ -1216,7 +1216,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-06 08:42:32</v>
+        <v>2026-10-07 08:06:59</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1228,9 +1228,9 @@
         <v/>
       </c>
       <c r="E2" t="str" xml:space="preserve">
-        <v xml:space="preserve">https://atomgit.com/openUBMC/website/issues/151
+        <v xml:space="preserve">https://gitcode.com/openUBMC/website/issues/151
 https://atomgit.com/openUBMC/website/issues/152
-https://gitcode.com/openUBMC/website/issues/153</v>
+https://atomgit.com/openUBMC/website/issues/153</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1326,7 +1326,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-06 08:42:32</v>
+        <v>2026-10-07 08:06:59</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1340,8 +1340,8 @@
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://gitcode.com/hifloat/hifloat-portal/issues/4
 https://gitcode.com/hifloat/hifloat-portal/issues/5
-https://atomgit.com/hifloat/hifloat-portal/issues/7
-https://atomgit.com/hifloat/hifloat-portal/issues/8</v>
+https://atomgit.com/hifloat/hifloat-portal/issues/6
+https://gitcode.com/hifloat/hifloat-portal/issues/7</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1356,7 +1356,7 @@
         <v>41</v>
       </c>
       <c r="J2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K2">
         <v>1</v>
@@ -1368,7 +1368,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O2">
         <v>0</v>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-10-08
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,7 +456,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-07 08:06:59</v>
+        <v>2026-10-08 08:23:36</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -564,7 +564,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-07 08:06:59</v>
+        <v>2026-10-08 08:23:36</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -672,7 +672,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-07 08:06:59</v>
+        <v>2026-10-08 08:23:36</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -780,20 +780,20 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-07 08:06:59</v>
+        <v>2026-10-08 08:23:36</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
       <c r="E2" t="str" xml:space="preserve">
-        <v xml:space="preserve">https://gitcode.com/opengauss/website/issues/404
-https://atomgit.com/opengauss/website/issues/367
+        <v xml:space="preserve">https://atomgit.com/opengauss/website/issues/404
+https://gitcode.com/opengauss/website/issues/367
 https://gitcode.com/opengauss/website/issues/360</v>
       </c>
       <c r="F2">
@@ -821,7 +821,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -890,7 +890,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-07 08:06:59</v>
+        <v>2026-10-08 08:23:36</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -998,7 +998,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-07 08:06:59</v>
+        <v>2026-10-08 08:23:36</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1106,7 +1106,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-07 08:06:59</v>
+        <v>2026-10-08 08:23:36</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1118,7 +1118,7 @@
         <v/>
       </c>
       <c r="E2" t="str" xml:space="preserve">
-        <v xml:space="preserve">https://atomgit.com/mindspore/mindspore-portal/issues/187
+        <v xml:space="preserve">https://gitcode.com/mindspore/mindspore-portal/issues/187
 https://gitcode.com/mindspore/mindspore-portal/issues/186
 https://gitcode.com/mindspore/mindspore-portal/issues/188</v>
       </c>
@@ -1216,7 +1216,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-07 08:06:59</v>
+        <v>2026-10-08 08:23:36</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1228,9 +1228,9 @@
         <v/>
       </c>
       <c r="E2" t="str" xml:space="preserve">
-        <v xml:space="preserve">https://gitcode.com/openUBMC/website/issues/151
+        <v xml:space="preserve">https://atomgit.com/openUBMC/website/issues/151
 https://atomgit.com/openUBMC/website/issues/152
-https://atomgit.com/openUBMC/website/issues/153</v>
+https://gitcode.com/openUBMC/website/issues/153</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1326,7 +1326,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-07 08:06:59</v>
+        <v>2026-10-08 08:23:36</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1338,10 +1338,10 @@
         <v/>
       </c>
       <c r="E2" t="str" xml:space="preserve">
-        <v xml:space="preserve">https://gitcode.com/hifloat/hifloat-portal/issues/4
-https://gitcode.com/hifloat/hifloat-portal/issues/5
-https://atomgit.com/hifloat/hifloat-portal/issues/6
-https://gitcode.com/hifloat/hifloat-portal/issues/7</v>
+        <v xml:space="preserve">https://atomgit.com/hifloat/hifloat-portal/issues/4
+https://atomgit.com/hifloat/hifloat-portal/issues/5
+https://gitcode.com/hifloat/hifloat-portal/issues/7
+https://gitcode.com/hifloat/hifloat-portal/issues/8</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1356,7 +1356,7 @@
         <v>41</v>
       </c>
       <c r="J2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K2">
         <v>1</v>
@@ -1368,7 +1368,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O2">
         <v>0</v>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-10-09
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,7 +456,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-08 08:23:36</v>
+        <v>2026-10-09 08:29:25</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -468,7 +468,7 @@
         <v/>
       </c>
       <c r="E2" t="str">
-        <v>https://gitcode.com/openeuler/openEuler-portal/issues/283</v>
+        <v>https://atomgit.com/openeuler/openEuler-portal/issues/283</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -564,7 +564,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-08 08:23:36</v>
+        <v>2026-10-09 08:29:25</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -672,7 +672,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-08 08:23:36</v>
+        <v>2026-10-09 08:29:25</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -780,21 +780,21 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-08 08:23:36</v>
+        <v>2026-10-09 08:29:25</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://atomgit.com/opengauss/website/issues/404
-https://gitcode.com/opengauss/website/issues/367
-https://gitcode.com/opengauss/website/issues/360</v>
+https://atomgit.com/opengauss/website/issues/367
+https://atomgit.com/opengauss/website/issues/360</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -821,7 +821,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -890,7 +890,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-08 08:23:36</v>
+        <v>2026-10-09 08:29:25</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -998,7 +998,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-08 08:23:36</v>
+        <v>2026-10-09 08:29:25</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1106,7 +1106,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-08 08:23:36</v>
+        <v>2026-10-09 08:29:25</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1118,9 +1118,9 @@
         <v/>
       </c>
       <c r="E2" t="str" xml:space="preserve">
-        <v xml:space="preserve">https://gitcode.com/mindspore/mindspore-portal/issues/187
-https://gitcode.com/mindspore/mindspore-portal/issues/186
-https://gitcode.com/mindspore/mindspore-portal/issues/188</v>
+        <v xml:space="preserve">https://atomgit.com/mindspore/mindspore-portal/issues/187
+https://atomgit.com/mindspore/mindspore-portal/issues/186
+https://atomgit.com/mindspore/mindspore-portal/issues/188</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1216,13 +1216,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-08 08:23:36</v>
+        <v>2026-10-09 08:29:25</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1230,7 +1230,7 @@
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://atomgit.com/openUBMC/website/issues/151
 https://atomgit.com/openUBMC/website/issues/152
-https://gitcode.com/openUBMC/website/issues/153</v>
+https://atomgit.com/openUBMC/website/issues/153</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1242,13 +1242,13 @@
         <v>2</v>
       </c>
       <c r="I2">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="L2">
         <v>0</v>
@@ -1326,13 +1326,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-08 08:23:36</v>
+        <v>2026-10-09 08:29:25</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1340,8 +1340,8 @@
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://atomgit.com/hifloat/hifloat-portal/issues/4
 https://atomgit.com/hifloat/hifloat-portal/issues/5
-https://gitcode.com/hifloat/hifloat-portal/issues/7
-https://gitcode.com/hifloat/hifloat-portal/issues/8</v>
+https://atomgit.com/hifloat/hifloat-portal/issues/6
+https://atomgit.com/hifloat/hifloat-portal/issues/7</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1356,7 +1356,7 @@
         <v>41</v>
       </c>
       <c r="J2">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K2">
         <v>1</v>
@@ -1368,7 +1368,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O2">
         <v>0</v>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-10-10
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,7 +456,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-09 08:29:25</v>
+        <v>2026-10-10 08:22:30</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -564,7 +564,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-09 08:29:25</v>
+        <v>2026-10-10 08:22:30</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -672,7 +672,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-09 08:29:25</v>
+        <v>2026-10-10 08:22:30</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -780,13 +780,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-09 08:29:25</v>
+        <v>2026-10-10 08:22:30</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -821,7 +821,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -890,7 +890,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-09 08:29:25</v>
+        <v>2026-10-10 08:22:30</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -998,7 +998,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-09 08:29:25</v>
+        <v>2026-10-10 08:22:30</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1106,13 +1106,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-09 08:29:25</v>
+        <v>2026-10-10 08:22:30</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1120,7 +1120,8 @@
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://atomgit.com/mindspore/mindspore-portal/issues/187
 https://atomgit.com/mindspore/mindspore-portal/issues/186
-https://atomgit.com/mindspore/mindspore-portal/issues/188</v>
+https://atomgit.com/mindspore/mindspore-portal/issues/188
+https://atomgit.com/mindspore/mindspore-portal/issues/267</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1132,7 +1133,7 @@
         <v>5</v>
       </c>
       <c r="I2">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="J2">
         <v>0</v>
@@ -1147,7 +1148,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -1216,13 +1217,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-09 08:29:25</v>
+        <v>2026-10-10 08:22:30</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1242,13 +1243,13 @@
         <v>2</v>
       </c>
       <c r="I2">
-        <v>41</v>
+        <v>10</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>147</v>
+        <v>179</v>
       </c>
       <c r="L2">
         <v>0</v>
@@ -1326,13 +1327,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-09 08:29:25</v>
+        <v>2026-10-10 08:22:30</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1356,7 +1357,7 @@
         <v>41</v>
       </c>
       <c r="J2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K2">
         <v>1</v>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-10-11
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,7 +456,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-10 08:22:30</v>
+        <v>2026-10-11 08:15:48</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -564,7 +564,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-10 08:22:30</v>
+        <v>2026-10-11 08:15:48</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -672,7 +672,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-10 08:22:30</v>
+        <v>2026-10-11 08:15:48</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -780,13 +780,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-10 08:22:30</v>
+        <v>2026-10-11 08:15:48</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -821,7 +821,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -890,7 +890,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-10 08:22:30</v>
+        <v>2026-10-11 08:15:48</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -998,7 +998,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-10 08:22:30</v>
+        <v>2026-10-11 08:15:48</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1106,13 +1106,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-10 08:22:30</v>
+        <v>2026-10-11 08:15:48</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1120,8 +1120,7 @@
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://atomgit.com/mindspore/mindspore-portal/issues/187
 https://atomgit.com/mindspore/mindspore-portal/issues/186
-https://atomgit.com/mindspore/mindspore-portal/issues/188
-https://atomgit.com/mindspore/mindspore-portal/issues/267</v>
+https://atomgit.com/mindspore/mindspore-portal/issues/188</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1148,7 +1147,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -1217,7 +1216,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-10 08:22:30</v>
+        <v>2026-10-11 08:15:48</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1327,43 +1326,42 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-10 08:22:30</v>
+        <v>2026-10-11 08:15:48</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>76</v>
+        <v>4</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
       <c r="E2" t="str" xml:space="preserve">
-        <v xml:space="preserve">https://atomgit.com/hifloat/hifloat-portal/issues/4
-https://atomgit.com/hifloat/hifloat-portal/issues/5
-https://atomgit.com/hifloat/hifloat-portal/issues/6
-https://atomgit.com/hifloat/hifloat-portal/issues/7</v>
+        <v xml:space="preserve">https://atomgit.com/hifloat/hifloat-portal/issues/28
+https://atomgit.com/hifloat/hifloat-portal/issues/29
+https://atomgit.com/hifloat/hifloat-portal/issues/30</v>
       </c>
       <c r="F2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H2">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="I2">
-        <v>41</v>
+        <v>0</v>
       </c>
       <c r="J2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L2">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M2">
         <v>0</v>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-10-12
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,7 +456,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-11 08:15:48</v>
+        <v>2026-10-12 08:31:39</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -564,7 +564,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-11 08:15:48</v>
+        <v>2026-10-12 08:31:39</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -672,7 +672,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-11 08:15:48</v>
+        <v>2026-10-12 08:31:39</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -780,7 +780,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-11 08:15:48</v>
+        <v>2026-10-12 08:31:39</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -890,7 +890,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-11 08:15:48</v>
+        <v>2026-10-12 08:31:39</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -998,7 +998,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-11 08:15:48</v>
+        <v>2026-10-12 08:31:39</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1106,7 +1106,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-11 08:15:48</v>
+        <v>2026-10-12 08:31:39</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1216,7 +1216,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-11 08:15:48</v>
+        <v>2026-10-12 08:31:39</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1326,42 +1326,43 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-11 08:15:48</v>
+        <v>2026-10-12 08:31:39</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>4</v>
+        <v>77</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
       <c r="E2" t="str" xml:space="preserve">
-        <v xml:space="preserve">https://atomgit.com/hifloat/hifloat-portal/issues/28
-https://atomgit.com/hifloat/hifloat-portal/issues/29
-https://atomgit.com/hifloat/hifloat-portal/issues/30</v>
+        <v xml:space="preserve">https://atomgit.com/hifloat/hifloat-portal/issues/4
+https://atomgit.com/hifloat/hifloat-portal/issues/5
+https://atomgit.com/hifloat/hifloat-portal/issues/6
+https://atomgit.com/hifloat/hifloat-portal/issues/7</v>
       </c>
       <c r="F2">
+        <v>0</v>
+      </c>
+      <c r="G2">
+        <v>0</v>
+      </c>
+      <c r="H2">
+        <v>33</v>
+      </c>
+      <c r="I2">
+        <v>41</v>
+      </c>
+      <c r="J2">
+        <v>2</v>
+      </c>
+      <c r="K2">
         <v>1</v>
       </c>
-      <c r="G2">
-        <v>1</v>
-      </c>
-      <c r="H2">
-        <v>0</v>
-      </c>
-      <c r="I2">
-        <v>0</v>
-      </c>
-      <c r="J2">
-        <v>0</v>
-      </c>
-      <c r="K2">
-        <v>0</v>
-      </c>
       <c r="L2">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M2">
         <v>0</v>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-10-13
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -454,21 +454,22 @@
         <v>tdk-schema-semantic</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-12 08:31:39</v>
+        <v>2026-10-13 09:07:53</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
-      <c r="E2" t="str">
-        <v>https://atomgit.com/openeuler/openEuler-portal/issues/283</v>
+      <c r="E2" t="str" xml:space="preserve">
+        <v xml:space="preserve">https://atomgit.com/openeuler/openEuler-portal/issues/283
+https://atomgit.com/openeuler/openEuler-portal/issues/335</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -495,7 +496,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -564,7 +565,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-12 08:31:39</v>
+        <v>2026-10-13 09:07:53</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -672,7 +673,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-12 08:31:39</v>
+        <v>2026-10-13 09:07:53</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -780,7 +781,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-12 08:31:39</v>
+        <v>2026-10-13 09:07:53</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -890,7 +891,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-12 08:31:39</v>
+        <v>2026-10-13 09:07:53</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -998,7 +999,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-12 08:31:39</v>
+        <v>2026-10-13 09:07:53</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1106,7 +1107,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-12 08:31:39</v>
+        <v>2026-10-13 09:07:53</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1216,13 +1217,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-12 08:31:39</v>
+        <v>2026-10-13 09:07:53</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>191</v>
+        <v>217</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1239,16 +1240,16 @@
         <v>0</v>
       </c>
       <c r="H2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I2">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>179</v>
+        <v>197</v>
       </c>
       <c r="L2">
         <v>0</v>
@@ -1326,13 +1327,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-12 08:31:39</v>
+        <v>2026-10-13 09:07:53</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1340,7 +1341,6 @@
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://atomgit.com/hifloat/hifloat-portal/issues/4
 https://atomgit.com/hifloat/hifloat-portal/issues/5
-https://atomgit.com/hifloat/hifloat-portal/issues/6
 https://atomgit.com/hifloat/hifloat-portal/issues/7</v>
       </c>
       <c r="F2">
@@ -1356,7 +1356,7 @@
         <v>41</v>
       </c>
       <c r="J2">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K2">
         <v>1</v>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-10-14
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -454,22 +454,21 @@
         <v>tdk-schema-semantic</v>
       </c>
     </row>
-    <row r="2" xml:space="preserve">
+    <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-13 09:07:53</v>
+        <v>2026-10-14 07:17:46</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
-      <c r="E2" t="str" xml:space="preserve">
-        <v xml:space="preserve">https://atomgit.com/openeuler/openEuler-portal/issues/283
-https://atomgit.com/openeuler/openEuler-portal/issues/335</v>
+      <c r="E2" t="str">
+        <v>https://atomgit.com/openeuler/openEuler-portal/issues/283</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -496,7 +495,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -565,7 +564,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-13 09:07:53</v>
+        <v>2026-10-14 07:17:46</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -673,7 +672,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-13 09:07:53</v>
+        <v>2026-10-14 07:17:46</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -781,13 +780,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-13 09:07:53</v>
+        <v>2026-10-14 07:17:46</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -822,7 +821,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -891,7 +890,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-13 09:07:53</v>
+        <v>2026-10-14 07:17:46</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -999,7 +998,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-13 09:07:53</v>
+        <v>2026-10-14 07:17:46</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1107,7 +1106,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-13 09:07:53</v>
+        <v>2026-10-14 07:17:46</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1217,13 +1216,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-13 09:07:53</v>
+        <v>2026-10-14 07:17:46</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>217</v>
+        <v>233</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1243,13 +1242,13 @@
         <v>3</v>
       </c>
       <c r="I2">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>197</v>
+        <v>206</v>
       </c>
       <c r="L2">
         <v>0</v>
@@ -1327,13 +1326,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-13 09:07:53</v>
+        <v>2026-10-14 07:17:46</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1341,6 +1340,7 @@
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://atomgit.com/hifloat/hifloat-portal/issues/4
 https://atomgit.com/hifloat/hifloat-portal/issues/5
+https://atomgit.com/hifloat/hifloat-portal/issues/6
 https://atomgit.com/hifloat/hifloat-portal/issues/7</v>
       </c>
       <c r="F2">
@@ -1356,7 +1356,7 @@
         <v>41</v>
       </c>
       <c r="J2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K2">
         <v>1</v>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-10-15
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -454,21 +454,22 @@
         <v>tdk-schema-semantic</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-14 07:17:46</v>
+        <v>2026-10-15 07:02:29</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
-      <c r="E2" t="str">
-        <v>https://atomgit.com/openeuler/openEuler-portal/issues/283</v>
+      <c r="E2" t="str" xml:space="preserve">
+        <v xml:space="preserve">https://atomgit.com/openeuler/openEuler-portal/issues/283
+https://atomgit.com/openeuler/openEuler-portal/issues/340</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -495,7 +496,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -564,7 +565,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-14 07:17:46</v>
+        <v>2026-10-15 07:02:29</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -672,7 +673,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-14 07:17:46</v>
+        <v>2026-10-15 07:02:29</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -780,13 +781,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-14 07:17:46</v>
+        <v>2026-10-15 07:02:29</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -821,7 +822,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -890,7 +891,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-14 07:17:46</v>
+        <v>2026-10-15 07:02:29</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -998,7 +999,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-14 07:17:46</v>
+        <v>2026-10-15 07:02:29</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1106,7 +1107,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-14 07:17:46</v>
+        <v>2026-10-15 07:02:29</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1216,13 +1217,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-14 07:17:46</v>
+        <v>2026-10-15 07:02:29</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1242,13 +1243,13 @@
         <v>3</v>
       </c>
       <c r="I2">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="L2">
         <v>0</v>
@@ -1326,13 +1327,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-14 07:17:46</v>
+        <v>2026-10-15 07:02:29</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>76</v>
+        <v>56</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1341,7 +1342,8 @@
         <v xml:space="preserve">https://atomgit.com/hifloat/hifloat-portal/issues/4
 https://atomgit.com/hifloat/hifloat-portal/issues/5
 https://atomgit.com/hifloat/hifloat-portal/issues/6
-https://atomgit.com/hifloat/hifloat-portal/issues/7</v>
+https://atomgit.com/hifloat/hifloat-portal/issues/7
+https://atomgit.com/hifloat/hifloat-portal/issues/8</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1350,10 +1352,10 @@
         <v>0</v>
       </c>
       <c r="H2">
-        <v>33</v>
+        <v>10</v>
       </c>
       <c r="I2">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -1368,7 +1370,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O2">
         <v>0</v>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-10-16
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -454,22 +454,21 @@
         <v>tdk-schema-semantic</v>
       </c>
     </row>
-    <row r="2" xml:space="preserve">
+    <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-15 07:02:29</v>
+        <v>2026-10-16 07:02:44</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
-      <c r="E2" t="str" xml:space="preserve">
-        <v xml:space="preserve">https://atomgit.com/openeuler/openEuler-portal/issues/283
-https://atomgit.com/openeuler/openEuler-portal/issues/340</v>
+      <c r="E2" t="str">
+        <v>https://atomgit.com/openeuler/openEuler-portal/issues/283</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -496,7 +495,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -565,7 +564,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-15 07:02:29</v>
+        <v>2026-10-16 07:02:44</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -673,7 +672,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-15 07:02:29</v>
+        <v>2026-10-16 07:02:44</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -781,13 +780,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-15 07:02:29</v>
+        <v>2026-10-16 07:02:44</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -822,7 +821,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -891,7 +890,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-15 07:02:29</v>
+        <v>2026-10-16 07:02:44</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -999,7 +998,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-15 07:02:29</v>
+        <v>2026-10-16 07:02:44</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1107,7 +1106,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-15 07:02:29</v>
+        <v>2026-10-16 07:02:44</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1217,7 +1216,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-15 07:02:29</v>
+        <v>2026-10-16 07:02:44</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1327,13 +1326,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-15 07:02:29</v>
+        <v>2026-10-16 07:02:44</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1342,8 +1341,7 @@
         <v xml:space="preserve">https://atomgit.com/hifloat/hifloat-portal/issues/4
 https://atomgit.com/hifloat/hifloat-portal/issues/5
 https://atomgit.com/hifloat/hifloat-portal/issues/6
-https://atomgit.com/hifloat/hifloat-portal/issues/7
-https://atomgit.com/hifloat/hifloat-portal/issues/8</v>
+https://atomgit.com/hifloat/hifloat-portal/issues/7</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1370,7 +1368,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O2">
         <v>0</v>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-10-17
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,7 +456,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-16 07:02:44</v>
+        <v>2026-10-17 06:36:12</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -564,7 +564,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-16 07:02:44</v>
+        <v>2026-10-17 06:36:12</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -672,7 +672,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-16 07:02:44</v>
+        <v>2026-10-17 06:36:12</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -780,7 +780,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-16 07:02:44</v>
+        <v>2026-10-17 06:36:12</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -890,7 +890,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-16 07:02:44</v>
+        <v>2026-10-17 06:36:12</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -998,7 +998,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-16 07:02:44</v>
+        <v>2026-10-17 06:36:12</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1106,7 +1106,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-16 07:02:44</v>
+        <v>2026-10-17 06:36:12</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1216,13 +1216,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-16 07:02:44</v>
+        <v>2026-10-17 06:36:12</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>235</v>
+        <v>223</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1242,13 +1242,13 @@
         <v>3</v>
       </c>
       <c r="I2">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>207</v>
+        <v>200</v>
       </c>
       <c r="L2">
         <v>0</v>
@@ -1326,13 +1326,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-16 07:02:44</v>
+        <v>2026-10-17 06:36:12</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1341,7 +1341,8 @@
         <v xml:space="preserve">https://atomgit.com/hifloat/hifloat-portal/issues/4
 https://atomgit.com/hifloat/hifloat-portal/issues/5
 https://atomgit.com/hifloat/hifloat-portal/issues/6
-https://atomgit.com/hifloat/hifloat-portal/issues/7</v>
+https://atomgit.com/hifloat/hifloat-portal/issues/7
+https://atomgit.com/hifloat/hifloat-portal/issues/8</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1368,7 +1369,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O2">
         <v>0</v>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-10-18
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,7 +456,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-17 06:36:12</v>
+        <v>2026-10-18 06:58:31</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -564,7 +564,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-17 06:36:12</v>
+        <v>2026-10-18 06:58:31</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -672,7 +672,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-17 06:36:12</v>
+        <v>2026-10-18 06:58:31</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -780,7 +780,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-17 06:36:12</v>
+        <v>2026-10-18 06:58:31</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -890,7 +890,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-17 06:36:12</v>
+        <v>2026-10-18 06:58:31</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -998,7 +998,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-17 06:36:12</v>
+        <v>2026-10-18 06:58:31</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1106,7 +1106,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-17 06:36:12</v>
+        <v>2026-10-18 06:58:31</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1216,7 +1216,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-17 06:36:12</v>
+        <v>2026-10-18 06:58:31</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1326,7 +1326,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-17 06:36:12</v>
+        <v>2026-10-18 06:58:31</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1357,7 +1357,7 @@
         <v>43</v>
       </c>
       <c r="J2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K2">
         <v>1</v>
@@ -1369,7 +1369,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O2">
         <v>0</v>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-10-19
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,7 +456,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-18 06:58:31</v>
+        <v>2026-10-19 07:18:31</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -564,7 +564,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-18 06:58:31</v>
+        <v>2026-10-19 07:18:31</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -672,7 +672,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-18 06:58:31</v>
+        <v>2026-10-19 07:18:31</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -780,13 +780,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-18 06:58:31</v>
+        <v>2026-10-19 07:18:31</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -821,7 +821,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -890,7 +890,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-18 06:58:31</v>
+        <v>2026-10-19 07:18:31</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -998,7 +998,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-18 06:58:31</v>
+        <v>2026-10-19 07:18:31</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1106,7 +1106,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-18 06:58:31</v>
+        <v>2026-10-19 07:18:31</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1216,13 +1216,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-18 06:58:31</v>
+        <v>2026-10-19 07:18:31</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1230,7 +1230,8 @@
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://atomgit.com/openUBMC/website/issues/151
 https://atomgit.com/openUBMC/website/issues/152
-https://atomgit.com/openUBMC/website/issues/153</v>
+https://atomgit.com/openUBMC/website/issues/153
+https://atomgit.com/openUBMC/website/issues/185</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1257,7 +1258,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -1326,13 +1327,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-18 06:58:31</v>
+        <v>2026-10-19 07:18:31</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1340,9 +1341,7 @@
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://atomgit.com/hifloat/hifloat-portal/issues/4
 https://atomgit.com/hifloat/hifloat-portal/issues/5
-https://atomgit.com/hifloat/hifloat-portal/issues/6
-https://atomgit.com/hifloat/hifloat-portal/issues/7
-https://atomgit.com/hifloat/hifloat-portal/issues/8</v>
+https://atomgit.com/hifloat/hifloat-portal/issues/7</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1357,7 +1356,7 @@
         <v>43</v>
       </c>
       <c r="J2">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K2">
         <v>1</v>
@@ -1369,7 +1368,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O2">
         <v>0</v>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-10-20
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,7 +456,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-19 07:18:31</v>
+        <v>2026-10-20 07:10:49</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -564,7 +564,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-19 07:18:31</v>
+        <v>2026-10-20 07:10:49</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -672,7 +672,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-19 07:18:31</v>
+        <v>2026-10-20 07:10:49</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -780,21 +780,20 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-19 07:18:31</v>
+        <v>2026-10-20 07:10:49</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://atomgit.com/opengauss/website/issues/404
-https://atomgit.com/opengauss/website/issues/367
-https://atomgit.com/opengauss/website/issues/360</v>
+https://atomgit.com/opengauss/website/issues/367</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -821,7 +820,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -890,7 +889,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-19 07:18:31</v>
+        <v>2026-10-20 07:10:49</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -998,7 +997,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-19 07:18:31</v>
+        <v>2026-10-20 07:10:49</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1106,13 +1105,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-19 07:18:31</v>
+        <v>2026-10-20 07:10:49</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1132,7 +1131,7 @@
         <v>5</v>
       </c>
       <c r="I2">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="J2">
         <v>0</v>
@@ -1216,13 +1215,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-19 07:18:31</v>
+        <v>2026-10-20 07:10:49</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>224</v>
+        <v>239</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1230,8 +1229,7 @@
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://atomgit.com/openUBMC/website/issues/151
 https://atomgit.com/openUBMC/website/issues/152
-https://atomgit.com/openUBMC/website/issues/153
-https://atomgit.com/openUBMC/website/issues/185</v>
+https://atomgit.com/openUBMC/website/issues/153</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1243,13 +1241,13 @@
         <v>3</v>
       </c>
       <c r="I2">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>200</v>
+        <v>209</v>
       </c>
       <c r="L2">
         <v>0</v>
@@ -1258,7 +1256,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -1327,13 +1325,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-19 07:18:31</v>
+        <v>2026-10-20 07:10:49</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1341,6 +1339,7 @@
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://atomgit.com/hifloat/hifloat-portal/issues/4
 https://atomgit.com/hifloat/hifloat-portal/issues/5
+https://atomgit.com/hifloat/hifloat-portal/issues/6
 https://atomgit.com/hifloat/hifloat-portal/issues/7</v>
       </c>
       <c r="F2">
@@ -1356,7 +1355,7 @@
         <v>43</v>
       </c>
       <c r="J2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K2">
         <v>1</v>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-10-21
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,7 +456,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-20 07:10:49</v>
+        <v>2026-10-21 07:03:38</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -564,7 +564,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-20 07:10:49</v>
+        <v>2026-10-21 07:03:38</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -672,7 +672,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-20 07:10:49</v>
+        <v>2026-10-21 07:03:38</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -780,20 +780,21 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-20 07:10:49</v>
+        <v>2026-10-21 07:03:38</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://atomgit.com/opengauss/website/issues/404
-https://atomgit.com/opengauss/website/issues/367</v>
+https://atomgit.com/opengauss/website/issues/367
+https://atomgit.com/opengauss/website/issues/442</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -820,7 +821,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -889,7 +890,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-20 07:10:49</v>
+        <v>2026-10-21 07:03:38</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -997,7 +998,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-20 07:10:49</v>
+        <v>2026-10-21 07:03:38</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1105,7 +1106,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-20 07:10:49</v>
+        <v>2026-10-21 07:03:38</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1215,7 +1216,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-20 07:10:49</v>
+        <v>2026-10-21 07:03:38</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1325,7 +1326,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-20 07:10:49</v>
+        <v>2026-10-21 07:03:38</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1339,8 +1340,8 @@
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://atomgit.com/hifloat/hifloat-portal/issues/4
 https://atomgit.com/hifloat/hifloat-portal/issues/5
-https://atomgit.com/hifloat/hifloat-portal/issues/6
-https://atomgit.com/hifloat/hifloat-portal/issues/7</v>
+https://atomgit.com/hifloat/hifloat-portal/issues/7
+https://atomgit.com/hifloat/hifloat-portal/issues/8</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1355,7 +1356,7 @@
         <v>43</v>
       </c>
       <c r="J2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K2">
         <v>1</v>
@@ -1367,7 +1368,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O2">
         <v>0</v>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-10-22
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -454,21 +454,22 @@
         <v>tdk-schema-semantic</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-21 07:03:38</v>
+        <v>2026-10-22 07:02:15</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
-      <c r="E2" t="str">
-        <v>https://atomgit.com/openeuler/openEuler-portal/issues/283</v>
+      <c r="E2" t="str" xml:space="preserve">
+        <v xml:space="preserve">https://atomgit.com/openeuler/openEuler-portal/issues/283
+https://atomgit.com/openeuler/openEuler-portal/issues/357</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -495,7 +496,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -564,7 +565,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-21 07:03:38</v>
+        <v>2026-10-22 07:02:15</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -672,7 +673,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-21 07:03:38</v>
+        <v>2026-10-22 07:02:15</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -780,13 +781,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-21 07:03:38</v>
+        <v>2026-10-22 07:02:15</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -821,7 +822,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -890,7 +891,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-21 07:03:38</v>
+        <v>2026-10-22 07:02:15</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -998,7 +999,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-21 07:03:38</v>
+        <v>2026-10-22 07:02:15</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1106,7 +1107,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-21 07:03:38</v>
+        <v>2026-10-22 07:02:15</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1216,13 +1217,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-21 07:03:38</v>
+        <v>2026-10-22 07:02:15</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1230,7 +1231,8 @@
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://atomgit.com/openUBMC/website/issues/151
 https://atomgit.com/openUBMC/website/issues/152
-https://atomgit.com/openUBMC/website/issues/153</v>
+https://atomgit.com/openUBMC/website/issues/153
+https://atomgit.com/openUBMC/website/issues/185</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1257,7 +1259,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -1326,25 +1328,26 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-10-21 07:03:38</v>
+        <v>2026-10-22 07:02:15</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
       <c r="E2" t="str" xml:space="preserve">
-        <v xml:space="preserve">https://atomgit.com/hifloat/hifloat-portal/issues/4
+        <v xml:space="preserve">https://atomgit.com/hifloat/hifloat-portal/issues/28
+https://atomgit.com/hifloat/hifloat-portal/issues/4
 https://atomgit.com/hifloat/hifloat-portal/issues/5
 https://atomgit.com/hifloat/hifloat-portal/issues/7
 https://atomgit.com/hifloat/hifloat-portal/issues/8</v>
       </c>
       <c r="F2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G2">
         <v>0</v>
@@ -1359,7 +1362,7 @@
         <v>0</v>
       </c>
       <c r="K2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L2">
         <v>0</v>

</xml_diff>